<commit_message>
Add Auto Expenses Only tab (fuel excluded)
Breaks the 97 non-fuel vehicle charges ($18,388.36) out of the combined
Fuel & Auto population, grouped into ten categories with per-card totals
and the exception flags carried through. Car washes are pulled in here
even where the tracker coded them as Fuel.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X9qK8zkdfoo6K5q1ScTX2U
</commit_message>
<xml_diff>
--- a/audit/Fuel_Auto_Fraud_Audit.xlsx
+++ b/audit/Fuel_Auto_Fraud_Audit.xlsx
@@ -13,10 +13,12 @@
     <sheet name="4. Vehicle Attribution" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5. Job Attribution" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6. Reconciliation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="7. Auto Expenses Only" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Flagged Transactions'!$A$1:$N$175</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3. Full Fuel &amp; Auto Ledger'!$A$1:$N$241</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'7. Auto Expenses Only'!$A$19:$J$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,11 +26,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="$#,##0.00;($#,##0.00);-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="DD-MMM-YY"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -161,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -233,6 +236,9 @@
     <xf numFmtId="164" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -25165,4 +25171,4357 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J117"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="56" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>AUTO EXPENSES ONLY — fuel excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Every vehicle-related charge that is not a pump/station fuel purchase. Car washes are included here even where the tracker coded them "Fuel".</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>SUMMARY BY CATEGORY</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Charges</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>AmEx $</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Capital One $</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Total $</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Of which flagged $</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="52" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="B6" s="52" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="53" t="n">
+        <v>3583.43</v>
+      </c>
+      <c r="D6" s="53" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E6" s="53" t="n">
+        <v>5983.43</v>
+      </c>
+      <c r="F6" s="53" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="55" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="B7" s="55" t="n">
+        <v>11</v>
+      </c>
+      <c r="C7" s="56" t="n">
+        <v>3390.41</v>
+      </c>
+      <c r="D7" s="56" t="n">
+        <v>1423.5</v>
+      </c>
+      <c r="E7" s="56" t="n">
+        <v>4813.91</v>
+      </c>
+      <c r="F7" s="56" t="n">
+        <v>4813.91</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="52" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="B8" s="52" t="n">
+        <v>8</v>
+      </c>
+      <c r="C8" s="53" t="n">
+        <v>1456.17</v>
+      </c>
+      <c r="D8" s="53" t="n">
+        <v>1079.65</v>
+      </c>
+      <c r="E8" s="53" t="n">
+        <v>2535.82</v>
+      </c>
+      <c r="F8" s="53" t="n">
+        <v>1125.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="52" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="B9" s="52" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="53" t="n">
+        <v>1692.92</v>
+      </c>
+      <c r="D9" s="53" t="n">
+        <v>12.95</v>
+      </c>
+      <c r="E9" s="53" t="n">
+        <v>1705.87</v>
+      </c>
+      <c r="F9" s="53" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="52" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="B10" s="52" t="n">
+        <v>18</v>
+      </c>
+      <c r="C10" s="53" t="n">
+        <v>545.66</v>
+      </c>
+      <c r="D10" s="53" t="n">
+        <v>479.94</v>
+      </c>
+      <c r="E10" s="53" t="n">
+        <v>1025.6</v>
+      </c>
+      <c r="F10" s="53" t="n">
+        <v>419.95</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="52" t="inlineStr">
+        <is>
+          <t>Towing</t>
+        </is>
+      </c>
+      <c r="B11" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="53" t="n">
+        <v>400</v>
+      </c>
+      <c r="D11" s="53" t="n">
+        <v>560</v>
+      </c>
+      <c r="E11" s="53" t="n">
+        <v>960</v>
+      </c>
+      <c r="F11" s="53" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="55" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="B12" s="55" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="56" t="n">
+        <v>491.95</v>
+      </c>
+      <c r="D12" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="56" t="n">
+        <v>491.95</v>
+      </c>
+      <c r="F12" s="56" t="n">
+        <v>491.95</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="55" t="inlineStr">
+        <is>
+          <t>Car rental</t>
+        </is>
+      </c>
+      <c r="B13" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="56" t="n">
+        <v>474.14</v>
+      </c>
+      <c r="D13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="56" t="n">
+        <v>474.14</v>
+      </c>
+      <c r="F13" s="56" t="n">
+        <v>474.14</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="52" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="B14" s="52" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" s="53" t="n">
+        <v>201.79</v>
+      </c>
+      <c r="D14" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="E14" s="53" t="n">
+        <v>217.79</v>
+      </c>
+      <c r="F14" s="53" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="55" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="B15" s="55" t="n">
+        <v>34</v>
+      </c>
+      <c r="C15" s="56" t="n">
+        <v>179.85</v>
+      </c>
+      <c r="D15" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="56" t="n">
+        <v>179.85</v>
+      </c>
+      <c r="F15" s="56" t="n">
+        <v>179.85</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="65" t="inlineStr">
+        <is>
+          <t>TOTAL AUTO EXPENSES</t>
+        </is>
+      </c>
+      <c r="B16" s="66" t="n">
+        <v>97</v>
+      </c>
+      <c r="C16" s="67" t="n">
+        <v>12416.32</v>
+      </c>
+      <c r="D16" s="67" t="n">
+        <v>5972.04</v>
+      </c>
+      <c r="E16" s="67" t="n">
+        <v>18388.36</v>
+      </c>
+      <c r="F16" s="67" t="n">
+        <v>9219.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>FULL DETAIL — 97 charges, newest last</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Description as booked</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Property / Job</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Company charged</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Source tab</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>Exception flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="n">
+        <v>45889</v>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>Equity Track – SFO prepaid parking</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr"/>
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I20" s="32" t="n">
+        <v>38</v>
+      </c>
+      <c r="J20" s="19" t="inlineStr">
+        <is>
+          <t>F9-FINE/VIOLATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="n">
+        <v>45893</v>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>Equity Track – SFO prepaid parking</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr"/>
+      <c r="G21" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I21" s="32" t="n">
+        <v>114</v>
+      </c>
+      <c r="J21" s="19" t="inlineStr">
+        <is>
+          <t>F9-FINE/VIOLATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="n">
+        <v>45894</v>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>Car rental</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>Enterprise Rent-A-Car</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>Travel – car rental (Mariaelena) - Equity Track</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr"/>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I22" s="32" t="n">
+        <v>474.14</v>
+      </c>
+      <c r="J22" s="19" t="inlineStr">
+        <is>
+          <t>F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="29" t="n">
+        <v>45895</v>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Bobcat of the Bay</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track – Bobcat supplies (hoses, couplers, hydraulic parts)</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr"/>
+      <c r="G23" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I23" s="30" t="n">
+        <v>517.89</v>
+      </c>
+      <c r="J23" s="16" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="n">
+        <v>45897</v>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track – car wash expense</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="inlineStr"/>
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I24" s="30" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="J24" s="16" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="n">
+        <v>45941</v>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing (Auto Pride)</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr"/>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I25" s="30" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="J25" s="16" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="31" t="n">
+        <v>45944</v>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>Equity Track – SFO prepaid parking</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr"/>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I26" s="32" t="n">
+        <v>38</v>
+      </c>
+      <c r="J26" s="19" t="inlineStr">
+        <is>
+          <t>F9-FINE/VIOLATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="n">
+        <v>45944</v>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="inlineStr"/>
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I27" s="30" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="J27" s="16" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="n">
+        <v>45945</v>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
+        <is>
+          <t>Equity Track – SFO prepaid parking</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr"/>
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H28" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I28" s="32" t="n">
+        <v>38</v>
+      </c>
+      <c r="J28" s="19" t="inlineStr">
+        <is>
+          <t>F9-FINE/VIOLATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="31" t="n">
+        <v>45945</v>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E29" s="19" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – parking citation/fine Juan's Mercedes</t>
+        </is>
+      </c>
+      <c r="F29" s="19" t="inlineStr"/>
+      <c r="G29" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H29" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I29" s="32" t="n">
+        <v>105.95</v>
+      </c>
+      <c r="J29" s="19" t="inlineStr">
+        <is>
+          <t>F9-FINE/VIOLATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="n">
+        <v>45958</v>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>Auto Expenses - Equity Track Inc</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="inlineStr"/>
+      <c r="G30" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I30" s="30" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="J30" s="16" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="29" t="n">
+        <v>45974</v>
+      </c>
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Beltran Tire Service</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – vehicle tire service/repair</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="inlineStr"/>
+      <c r="G31" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I31" s="30" t="n">
+        <v>1140.03</v>
+      </c>
+      <c r="J31" s="16" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="29" t="n">
+        <v>45975</v>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="inlineStr"/>
+      <c r="G32" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I32" s="30" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="J32" s="16" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="29" t="n">
+        <v>45975</v>
+      </c>
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>BTPeragon Enterprises</t>
+        </is>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – truck bed cover (BTperagon)</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="inlineStr"/>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I33" s="30" t="n">
+        <v>1530.16</v>
+      </c>
+      <c r="J33" s="16" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="29" t="n">
+        <v>45975</v>
+      </c>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>Logiq Air Suspension Solutions</t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – air suspension remote (Logiq Air system)</t>
+        </is>
+      </c>
+      <c r="F34" s="16" t="inlineStr"/>
+      <c r="G34" s="16" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="H34" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I34" s="30" t="n">
+        <v>174.01</v>
+      </c>
+      <c r="J34" s="16" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="n">
+        <v>45975</v>
+      </c>
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Logiq Air Suspension Solutions</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – truck air suspension kit (Logiq Air)</t>
+        </is>
+      </c>
+      <c r="F35" s="16" t="inlineStr"/>
+      <c r="G35" s="16" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I35" s="30" t="n">
+        <v>1879.26</v>
+      </c>
+      <c r="J35" s="16" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="31" t="n">
+        <v>45976</v>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – airport parking/terminal expense (San Jose)</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr"/>
+      <c r="G36" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H36" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I36" s="32" t="n">
+        <v>50</v>
+      </c>
+      <c r="J36" s="19" t="inlineStr">
+        <is>
+          <t>F9-FINE/VIOLATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="n">
+        <v>45983</v>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing</t>
+        </is>
+      </c>
+      <c r="F37" s="16" t="inlineStr"/>
+      <c r="G37" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I37" s="30" t="n">
+        <v>79.98999999999999</v>
+      </c>
+      <c r="J37" s="16" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="29" t="n">
+        <v>45989</v>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="inlineStr"/>
+      <c r="G38" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H38" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I38" s="30" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="J38" s="16" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="29" t="n">
+        <v>45999</v>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>CA DMV</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – DMV vehicle filing/processing fee</t>
+        </is>
+      </c>
+      <c r="F39" s="16" t="inlineStr"/>
+      <c r="G39" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H39" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I39" s="30" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="J39" s="16" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="29" t="n">
+        <v>45999</v>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>CA DMV</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – DMV vehicle registration/service fee</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr"/>
+      <c r="G40" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H40" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I40" s="30" t="n">
+        <v>509</v>
+      </c>
+      <c r="J40" s="16" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="29" t="n">
+        <v>46005</v>
+      </c>
+      <c r="B41" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E41" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing</t>
+        </is>
+      </c>
+      <c r="F41" s="16" t="inlineStr"/>
+      <c r="G41" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H41" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I41" s="30" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="J41" s="16" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="29" t="n">
+        <v>46008</v>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>CA DMV</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle registration or DMV fee</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="inlineStr"/>
+      <c r="G42" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H42" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I42" s="30" t="n">
+        <v>17.04</v>
+      </c>
+      <c r="J42" s="16" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="29" t="n">
+        <v>46008</v>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>State of California</t>
+        </is>
+      </c>
+      <c r="E43" s="16" t="inlineStr">
+        <is>
+          <t>DMV payment (license/registration)</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="inlineStr"/>
+      <c r="G43" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H43" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I43" s="30" t="n">
+        <v>874</v>
+      </c>
+      <c r="J43" s="16" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="29" t="n">
+        <v>46013</v>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>Car wash</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr"/>
+      <c r="G44" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H44" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I44" s="30" t="n">
+        <v>79.98999999999999</v>
+      </c>
+      <c r="J44" s="16" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="31" t="n">
+        <v>46014</v>
+      </c>
+      <c r="B45" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C45" s="19" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D45" s="19" t="inlineStr">
+        <is>
+          <t>CA DMV</t>
+        </is>
+      </c>
+      <c r="E45" s="19" t="inlineStr">
+        <is>
+          <t>Vehicle registration or DMV fee - Lucas's DMV Schedule</t>
+        </is>
+      </c>
+      <c r="F45" s="19" t="inlineStr"/>
+      <c r="G45" s="19" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H45" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I45" s="32" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J45" s="19" t="inlineStr">
+        <is>
+          <t>F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="31" t="n">
+        <v>46014</v>
+      </c>
+      <c r="B46" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C46" s="19" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D46" s="19" t="inlineStr">
+        <is>
+          <t>CA DMV</t>
+        </is>
+      </c>
+      <c r="E46" s="19" t="inlineStr">
+        <is>
+          <t>Vehicle registration or DMV fee - Lucas's DMV Schedule</t>
+        </is>
+      </c>
+      <c r="F46" s="19" t="inlineStr"/>
+      <c r="G46" s="19" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H46" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I46" s="32" t="n">
+        <v>45</v>
+      </c>
+      <c r="J46" s="19" t="inlineStr">
+        <is>
+          <t>F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="29" t="n">
+        <v>46019</v>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>Car wash</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="inlineStr"/>
+      <c r="G47" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H47" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I47" s="30" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="J47" s="16" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="33" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C48" s="22" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D48" s="22" t="inlineStr">
+        <is>
+          <t>FASTRAK</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="inlineStr">
+        <is>
+          <t>FASTRAK</t>
+        </is>
+      </c>
+      <c r="F48" s="22" t="inlineStr"/>
+      <c r="G48" s="22" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H48" s="22" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I48" s="34" t="n">
+        <v>580</v>
+      </c>
+      <c r="J48" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F9-BULK TOLL, NO VEHICLE NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="29" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>SQ *GOLDEN STATE WRAPS</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>PPS - Van Wrap payment</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="inlineStr"/>
+      <c r="G49" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="H49" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I49" s="30" t="n">
+        <v>1200</v>
+      </c>
+      <c r="J49" s="16" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="33" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D50" s="22" t="inlineStr">
+        <is>
+          <t>FASTRAK</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="inlineStr">
+        <is>
+          <t>All Vehicles</t>
+        </is>
+      </c>
+      <c r="F50" s="22" t="inlineStr"/>
+      <c r="G50" s="22" t="inlineStr">
+        <is>
+          <t>Equity Track 8251</t>
+        </is>
+      </c>
+      <c r="H50" s="22" t="inlineStr">
+        <is>
+          <t>Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I50" s="34" t="n">
+        <v>580</v>
+      </c>
+      <c r="J50" s="22" t="inlineStr">
+        <is>
+          <t>F1-DUPLICATE POSTING; F6-UNCATEGORISED (blank bucket); F9-BULK TOLL, NO VEHICLE NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="33" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B51" s="22" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="D51" s="22" t="inlineStr">
+        <is>
+          <t>SQ *GOLDEN STATE WRAPS</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="inlineStr">
+        <is>
+          <t>PPS - Van Wrap - Peninsula Plumbing Solution</t>
+        </is>
+      </c>
+      <c r="F51" s="22" t="inlineStr"/>
+      <c r="G51" s="22" t="inlineStr">
+        <is>
+          <t>PPS Relay</t>
+        </is>
+      </c>
+      <c r="H51" s="22" t="inlineStr">
+        <is>
+          <t>PPS Expenses</t>
+        </is>
+      </c>
+      <c r="I51" s="34" t="n">
+        <v>1200</v>
+      </c>
+      <c r="J51" s="22" t="inlineStr">
+        <is>
+          <t>F1-DUPLICATE POSTING; F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="29" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash Subscription</t>
+        </is>
+      </c>
+      <c r="F52" s="16" t="inlineStr"/>
+      <c r="G52" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H52" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I52" s="30" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="J52" s="16" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="33" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B53" s="22" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C53" s="22" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D53" s="22" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E53" s="22" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash Subscription</t>
+        </is>
+      </c>
+      <c r="F53" s="22" t="inlineStr"/>
+      <c r="G53" s="22" t="inlineStr">
+        <is>
+          <t>Equity Track 8251</t>
+        </is>
+      </c>
+      <c r="H53" s="22" t="inlineStr">
+        <is>
+          <t>Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I53" s="34" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="J53" s="22" t="inlineStr">
+        <is>
+          <t>F1-DUPLICATE POSTING; F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="29" t="n">
+        <v>46064</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>MTA Meter</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>MTA Parking Meter Fee</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="inlineStr"/>
+      <c r="G54" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H54" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I54" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="J54" s="16" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="31" t="n">
+        <v>46064</v>
+      </c>
+      <c r="B55" s="19" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C55" s="19" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>TCB*MTA METER MTA MCK</t>
+        </is>
+      </c>
+      <c r="E55" s="19" t="inlineStr">
+        <is>
+          <t>Parking Meters</t>
+        </is>
+      </c>
+      <c r="F55" s="19" t="inlineStr"/>
+      <c r="G55" s="19" t="inlineStr">
+        <is>
+          <t>Equity Track 8251</t>
+        </is>
+      </c>
+      <c r="H55" s="19" t="inlineStr">
+        <is>
+          <t>Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I55" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="J55" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="29" t="n">
+        <v>46070</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>Towing</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Loural Towing</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="inlineStr">
+        <is>
+          <t>Drop off Ford F350</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr"/>
+      <c r="G56" s="16" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="H56" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I56" s="30" t="n">
+        <v>280</v>
+      </c>
+      <c r="J56" s="16" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="33" t="n">
+        <v>46070</v>
+      </c>
+      <c r="B57" s="22" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>Towing</t>
+        </is>
+      </c>
+      <c r="D57" s="22" t="inlineStr">
+        <is>
+          <t>SQ*LOURAL TOWING</t>
+        </is>
+      </c>
+      <c r="E57" s="22" t="inlineStr">
+        <is>
+          <t>Drop off Ford F350</t>
+        </is>
+      </c>
+      <c r="F57" s="22" t="inlineStr"/>
+      <c r="G57" s="22" t="inlineStr">
+        <is>
+          <t>Equity Track 8251</t>
+        </is>
+      </c>
+      <c r="H57" s="22" t="inlineStr">
+        <is>
+          <t>Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I57" s="34" t="n">
+        <v>280</v>
+      </c>
+      <c r="J57" s="22" t="inlineStr">
+        <is>
+          <t>F1-DUPLICATE POSTING; F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="29" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>Towing</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>City Towing</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr"/>
+      <c r="F58" s="16" t="inlineStr">
+        <is>
+          <t>1202 Via Lucas</t>
+        </is>
+      </c>
+      <c r="G58" s="16" t="inlineStr">
+        <is>
+          <t>Relay 5776</t>
+        </is>
+      </c>
+      <c r="H58" s="16" t="inlineStr">
+        <is>
+          <t>Property Expenses</t>
+        </is>
+      </c>
+      <c r="I58" s="30" t="n">
+        <v>400</v>
+      </c>
+      <c r="J58" s="16" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="31" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B59" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>LAZ PARKING</t>
+        </is>
+      </c>
+      <c r="E59" s="19" t="inlineStr"/>
+      <c r="F59" s="19" t="inlineStr"/>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I59" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="J59" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="31" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B60" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>FASTRAK</t>
+        </is>
+      </c>
+      <c r="E60" s="19" t="inlineStr"/>
+      <c r="F60" s="19" t="inlineStr">
+        <is>
+          <t>100 Palm Ave</t>
+        </is>
+      </c>
+      <c r="G60" s="19" t="inlineStr">
+        <is>
+          <t>Equity Track 8251</t>
+        </is>
+      </c>
+      <c r="H60" s="19" t="inlineStr">
+        <is>
+          <t>Property Expenses</t>
+        </is>
+      </c>
+      <c r="I60" s="32" t="n">
+        <v>327.91</v>
+      </c>
+      <c r="J60" s="19" t="inlineStr">
+        <is>
+          <t>F9-BULK TOLL, NO VEHICLE NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="31" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B61" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>FASTRAK</t>
+        </is>
+      </c>
+      <c r="E61" s="19" t="inlineStr"/>
+      <c r="F61" s="19" t="inlineStr">
+        <is>
+          <t>Split Properties</t>
+        </is>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Equity Track 8251</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>Property Expenses</t>
+        </is>
+      </c>
+      <c r="I61" s="32" t="n">
+        <v>580</v>
+      </c>
+      <c r="J61" s="19" t="inlineStr">
+        <is>
+          <t>F9-BULK TOLL, NO VEHICLE NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="31" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B62" s="19" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C62" s="19" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E62" s="19" t="inlineStr"/>
+      <c r="F62" s="19" t="inlineStr"/>
+      <c r="G62" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H62" s="19" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I62" s="32" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="J62" s="19" t="inlineStr">
+        <is>
+          <t>F8-MISCODED AS FUEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="31" t="n">
+        <v>46094</v>
+      </c>
+      <c r="B63" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>SFMTA CIT PYMNT WEB</t>
+        </is>
+      </c>
+      <c r="E63" s="19" t="inlineStr"/>
+      <c r="F63" s="19" t="inlineStr"/>
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I63" s="32" t="n">
+        <v>108</v>
+      </c>
+      <c r="J63" s="19" t="inlineStr">
+        <is>
+          <t>F9-FINE/VIOLATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="29" t="n">
+        <v>46100</v>
+      </c>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>MTA METERS - MTA PBP</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
+          <t>Parking Payment for Alan</t>
+        </is>
+      </c>
+      <c r="F64" s="16" t="inlineStr"/>
+      <c r="G64" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="H64" s="16" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I64" s="30" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="J64" s="16" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="33" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B65" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C65" s="22" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D65" s="22" t="inlineStr">
+        <is>
+          <t>Fastrak</t>
+        </is>
+      </c>
+      <c r="E65" s="22" t="inlineStr"/>
+      <c r="F65" s="22" t="inlineStr"/>
+      <c r="G65" s="22" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H65" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I65" s="34" t="n">
+        <v>255</v>
+      </c>
+      <c r="J65" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F9-BULK TOLL, NO VEHICLE NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="31" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B66" s="19" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C66" s="19" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D66" s="19" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E66" s="19" t="inlineStr"/>
+      <c r="F66" s="19" t="inlineStr"/>
+      <c r="G66" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H66" s="19" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I66" s="32" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="J66" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="33" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B67" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C67" s="22" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D67" s="22" t="inlineStr">
+        <is>
+          <t>FASTRAK VIOLATION CESAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E67" s="22" t="inlineStr"/>
+      <c r="F67" s="22" t="inlineStr"/>
+      <c r="G67" s="22" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H67" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I67" s="34" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="J67" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F9-FINE/VIOLATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="33" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B68" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C68" s="22" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D68" s="22" t="inlineStr">
+        <is>
+          <t>FASTRAK CSC TOLLS OAKLAND CA</t>
+        </is>
+      </c>
+      <c r="E68" s="22" t="inlineStr"/>
+      <c r="F68" s="22" t="inlineStr"/>
+      <c r="G68" s="22" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H68" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I68" s="34" t="n">
+        <v>700</v>
+      </c>
+      <c r="J68" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F9-BULK TOLL, NO VEHICLE NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="31" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B69" s="19" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C69" s="19" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D69" s="19" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E69" s="19" t="inlineStr"/>
+      <c r="F69" s="19" t="inlineStr"/>
+      <c r="G69" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H69" s="19" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I69" s="32" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="J69" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="33" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B70" s="22" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C70" s="22" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D70" s="22" t="inlineStr">
+        <is>
+          <t>State of California DMV</t>
+        </is>
+      </c>
+      <c r="E70" s="22" t="inlineStr"/>
+      <c r="F70" s="22" t="inlineStr"/>
+      <c r="G70" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H70" s="22" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="I70" s="34" t="n">
+        <v>1059</v>
+      </c>
+      <c r="J70" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="33" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B71" s="22" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C71" s="22" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D71" s="22" t="inlineStr">
+        <is>
+          <t>DMV Fee</t>
+        </is>
+      </c>
+      <c r="E71" s="22" t="inlineStr"/>
+      <c r="F71" s="22" t="inlineStr"/>
+      <c r="G71" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H71" s="22" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="I71" s="34" t="n">
+        <v>20.65</v>
+      </c>
+      <c r="J71" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="29" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B72" s="16" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C72" s="16" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="D72" s="16" t="inlineStr">
+        <is>
+          <t>Autozone</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr"/>
+      <c r="F72" s="16" t="inlineStr">
+        <is>
+          <t>820 28th St</t>
+        </is>
+      </c>
+      <c r="G72" s="16" t="inlineStr"/>
+      <c r="H72" s="16" t="inlineStr">
+        <is>
+          <t>Capital One Business Property E</t>
+        </is>
+      </c>
+      <c r="I72" s="30" t="n">
+        <v>12.95</v>
+      </c>
+      <c r="J72" s="16" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="31" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B73" s="19" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C73" s="19" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D73" s="19" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E73" s="19" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="F73" s="19" t="inlineStr"/>
+      <c r="G73" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H73" s="19" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I73" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="J73" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="33" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B74" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C74" s="22" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D74" s="22" t="inlineStr">
+        <is>
+          <t>FASTRAK VIOLATION CESAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E74" s="22" t="inlineStr"/>
+      <c r="F74" s="22" t="inlineStr"/>
+      <c r="G74" s="22" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H74" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I74" s="34" t="n">
+        <v>102</v>
+      </c>
+      <c r="J74" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F9-FINE/VIOLATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="33" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B75" s="22" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C75" s="22" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D75" s="22" t="inlineStr">
+        <is>
+          <t>FasTrak</t>
+        </is>
+      </c>
+      <c r="E75" s="22" t="inlineStr"/>
+      <c r="F75" s="22" t="inlineStr"/>
+      <c r="G75" s="22" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="H75" s="22" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="I75" s="34" t="n">
+        <v>263.5</v>
+      </c>
+      <c r="J75" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F9-BULK TOLL, NO VEHICLE NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="33" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B76" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C76" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D76" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E76" s="22" t="inlineStr"/>
+      <c r="F76" s="22" t="inlineStr"/>
+      <c r="G76" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H76" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I76" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J76" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="33" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B77" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C77" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D77" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E77" s="22" t="inlineStr"/>
+      <c r="F77" s="22" t="inlineStr"/>
+      <c r="G77" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H77" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I77" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J77" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="33" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B78" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C78" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D78" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E78" s="22" t="inlineStr"/>
+      <c r="F78" s="22" t="inlineStr"/>
+      <c r="G78" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H78" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I78" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J78" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="33" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B79" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C79" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D79" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E79" s="22" t="inlineStr"/>
+      <c r="F79" s="22" t="inlineStr"/>
+      <c r="G79" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H79" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I79" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J79" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="33" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B80" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C80" s="22" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D80" s="22" t="inlineStr">
+        <is>
+          <t>FASTRAK CSC TOLLS</t>
+        </is>
+      </c>
+      <c r="E80" s="22" t="inlineStr"/>
+      <c r="F80" s="22" t="inlineStr"/>
+      <c r="G80" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H80" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I80" s="34" t="n">
+        <v>700</v>
+      </c>
+      <c r="J80" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY); F9-BULK TOLL, NO VEHICLE NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="33" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B81" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C81" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D81" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E81" s="22" t="inlineStr"/>
+      <c r="F81" s="22" t="inlineStr"/>
+      <c r="G81" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H81" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I81" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J81" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="33" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B82" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C82" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D82" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E82" s="22" t="inlineStr"/>
+      <c r="F82" s="22" t="inlineStr"/>
+      <c r="G82" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H82" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I82" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J82" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="33" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B83" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C83" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D83" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E83" s="22" t="inlineStr"/>
+      <c r="F83" s="22" t="inlineStr"/>
+      <c r="G83" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H83" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I83" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J83" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="33" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B84" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C84" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D84" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E84" s="22" t="inlineStr"/>
+      <c r="F84" s="22" t="inlineStr"/>
+      <c r="G84" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H84" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I84" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J84" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="31" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B85" s="19" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C85" s="19" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D85" s="19" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E85" s="19" t="inlineStr"/>
+      <c r="F85" s="19" t="inlineStr"/>
+      <c r="G85" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H85" s="19" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I85" s="32" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="J85" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="33" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B86" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C86" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D86" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E86" s="22" t="inlineStr"/>
+      <c r="F86" s="22" t="inlineStr"/>
+      <c r="G86" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H86" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I86" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J86" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="31" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B87" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C87" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D87" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E87" s="19" t="inlineStr"/>
+      <c r="F87" s="19" t="inlineStr"/>
+      <c r="G87" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H87" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I87" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J87" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="31" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B88" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C88" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D88" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E88" s="19" t="inlineStr"/>
+      <c r="F88" s="19" t="inlineStr"/>
+      <c r="G88" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H88" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I88" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J88" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="31" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B89" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C89" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D89" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E89" s="19" t="inlineStr"/>
+      <c r="F89" s="19" t="inlineStr"/>
+      <c r="G89" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H89" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I89" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J89" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="31" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B90" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D90" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E90" s="19" t="inlineStr"/>
+      <c r="F90" s="19" t="inlineStr"/>
+      <c r="G90" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H90" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I90" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J90" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="33" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B91" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C91" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D91" s="22" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E91" s="22" t="inlineStr"/>
+      <c r="F91" s="22" t="inlineStr"/>
+      <c r="G91" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H91" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I91" s="34" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="J91" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="31" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B92" s="19" t="inlineStr">
+        <is>
+          <t>Capital One</t>
+        </is>
+      </c>
+      <c r="C92" s="19" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D92" s="19" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E92" s="19" t="inlineStr"/>
+      <c r="F92" s="19" t="inlineStr"/>
+      <c r="G92" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H92" s="19" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I92" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="J92" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="33" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B93" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C93" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D93" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E93" s="22" t="inlineStr"/>
+      <c r="F93" s="22" t="inlineStr"/>
+      <c r="G93" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H93" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I93" s="34" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="J93" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="33" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B94" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C94" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D94" s="22" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E94" s="22" t="inlineStr"/>
+      <c r="F94" s="22" t="inlineStr"/>
+      <c r="G94" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H94" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I94" s="34" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J94" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="33" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B95" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C95" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D95" s="22" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E95" s="22" t="inlineStr"/>
+      <c r="F95" s="22" t="inlineStr"/>
+      <c r="G95" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H95" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I95" s="34" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="J95" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="31" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B96" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D96" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER PHONESAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E96" s="19" t="inlineStr"/>
+      <c r="F96" s="19" t="inlineStr"/>
+      <c r="G96" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H96" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I96" s="32" t="n">
+        <v>-2.05</v>
+      </c>
+      <c r="J96" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="33" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B97" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C97" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D97" s="22" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E97" s="22" t="inlineStr"/>
+      <c r="F97" s="22" t="inlineStr"/>
+      <c r="G97" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H97" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I97" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J97" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="33" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B98" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C98" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D98" s="22" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E98" s="22" t="inlineStr"/>
+      <c r="F98" s="22" t="inlineStr"/>
+      <c r="G98" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H98" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I98" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J98" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="31" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B99" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C99" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D99" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E99" s="19" t="inlineStr"/>
+      <c r="F99" s="19" t="inlineStr"/>
+      <c r="G99" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H99" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I99" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J99" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="31" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B100" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C100" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D100" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E100" s="19" t="inlineStr"/>
+      <c r="F100" s="19" t="inlineStr"/>
+      <c r="G100" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H100" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I100" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J100" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="33" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B101" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C101" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D101" s="22" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO       CA</t>
+        </is>
+      </c>
+      <c r="E101" s="22" t="inlineStr"/>
+      <c r="F101" s="22" t="inlineStr"/>
+      <c r="G101" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H101" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I101" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J101" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="33" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B102" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C102" s="22" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D102" s="22" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO       CA</t>
+        </is>
+      </c>
+      <c r="E102" s="22" t="inlineStr"/>
+      <c r="F102" s="22" t="inlineStr"/>
+      <c r="G102" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H102" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I102" s="34" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J102" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="31" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B103" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C103" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D103" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANC</t>
+        </is>
+      </c>
+      <c r="E103" s="19" t="inlineStr"/>
+      <c r="F103" s="19" t="inlineStr"/>
+      <c r="G103" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H103" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I103" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J103" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="31" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B104" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C104" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D104" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANC</t>
+        </is>
+      </c>
+      <c r="E104" s="19" t="inlineStr"/>
+      <c r="F104" s="19" t="inlineStr"/>
+      <c r="G104" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H104" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I104" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J104" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="31" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B105" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C105" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D105" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E105" s="19" t="inlineStr"/>
+      <c r="F105" s="19" t="inlineStr"/>
+      <c r="G105" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H105" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I105" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J105" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="31" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B106" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C106" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D106" s="19" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E106" s="19" t="inlineStr"/>
+      <c r="F106" s="19" t="inlineStr"/>
+      <c r="G106" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H106" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I106" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J106" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="31" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B107" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C107" s="19" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="D107" s="19" t="inlineStr">
+        <is>
+          <t>BELTRAN TIRES INC - REDWOOD CITY CA</t>
+        </is>
+      </c>
+      <c r="E107" s="19" t="inlineStr"/>
+      <c r="F107" s="19" t="inlineStr"/>
+      <c r="G107" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H107" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I107" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="J107" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="33" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B108" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C108" s="22" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D108" s="22" t="inlineStr">
+        <is>
+          <t>82858 - TERMINAL A ESAN JOSE CA</t>
+        </is>
+      </c>
+      <c r="E108" s="22" t="inlineStr"/>
+      <c r="F108" s="22" t="inlineStr"/>
+      <c r="G108" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H108" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I108" s="34" t="n">
+        <v>75</v>
+      </c>
+      <c r="J108" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="33" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B109" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C109" s="22" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D109" s="22" t="inlineStr">
+        <is>
+          <t>60774 - SFO PARKING SAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E109" s="22" t="inlineStr"/>
+      <c r="F109" s="22" t="inlineStr"/>
+      <c r="G109" s="22" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="H109" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I109" s="34" t="n">
+        <v>111</v>
+      </c>
+      <c r="J109" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="31" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B110" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C110" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D110" s="19" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E110" s="19" t="inlineStr"/>
+      <c r="F110" s="19" t="inlineStr"/>
+      <c r="G110" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H110" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I110" s="32" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="J110" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="33" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B111" s="22" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C111" s="22" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D111" s="22" t="inlineStr">
+        <is>
+          <t>FASTRAK</t>
+        </is>
+      </c>
+      <c r="E111" s="22" t="inlineStr"/>
+      <c r="F111" s="22" t="inlineStr"/>
+      <c r="G111" s="22" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H111" s="22" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I111" s="34" t="n">
+        <v>700</v>
+      </c>
+      <c r="J111" s="22" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F9-BULK TOLL, NO VEHICLE NAMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="31" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B112" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C112" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D112" s="19" t="inlineStr">
+        <is>
+          <t>Clipper Trans</t>
+        </is>
+      </c>
+      <c r="E112" s="19" t="inlineStr"/>
+      <c r="F112" s="19" t="inlineStr"/>
+      <c r="G112" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H112" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I112" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J112" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="31" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B113" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C113" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D113" s="19" t="inlineStr">
+        <is>
+          <t>Clipper Trans</t>
+        </is>
+      </c>
+      <c r="E113" s="19" t="inlineStr"/>
+      <c r="F113" s="19" t="inlineStr"/>
+      <c r="G113" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H113" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I113" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J113" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="31" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B114" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C114" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D114" s="19" t="inlineStr">
+        <is>
+          <t>Clipper Trans</t>
+        </is>
+      </c>
+      <c r="E114" s="19" t="inlineStr"/>
+      <c r="F114" s="19" t="inlineStr"/>
+      <c r="G114" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H114" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I114" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J114" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="31" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B115" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C115" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D115" s="19" t="inlineStr">
+        <is>
+          <t>Clipper Trans</t>
+        </is>
+      </c>
+      <c r="E115" s="19" t="inlineStr"/>
+      <c r="F115" s="19" t="inlineStr"/>
+      <c r="G115" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H115" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I115" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J115" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="31" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B116" s="19" t="inlineStr">
+        <is>
+          <t>AmEx</t>
+        </is>
+      </c>
+      <c r="C116" s="19" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D116" s="19" t="inlineStr">
+        <is>
+          <t>Clipper Trans</t>
+        </is>
+      </c>
+      <c r="E116" s="19" t="inlineStr"/>
+      <c r="F116" s="19" t="inlineStr"/>
+      <c r="G116" s="19" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="H116" s="19" t="inlineStr">
+        <is>
+          <t>Copy of Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="I116" s="32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="J116" s="19" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="H117" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="I117" s="35" t="n">
+        <v>18388.36</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A19:J116"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Auto by Company tab and resolve the Capital One $230 question
Groups the 92 de-duplicated auto charges ($16,260.37) by entity with a
company x category matrix and a per-card split. Five Capital One rows
that appear on two tabs each ($2,127.99) are now counted once, under the
entity their twin names.

Also documents the search for Capital One's $230: no cell, subtotal or
row combination in the tracker produces it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X9qK8zkdfoo6K5q1ScTX2U
</commit_message>
<xml_diff>
--- a/audit/Fuel_Auto_Fraud_Audit.xlsx
+++ b/audit/Fuel_Auto_Fraud_Audit.xlsx
@@ -14,6 +14,7 @@
     <sheet name="5. Job Attribution" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6. Reconciliation" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="7. Auto Expenses Only" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="8. Auto by Company" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Flagged Transactions'!$A$1:$N$175</definedName>
@@ -164,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -239,6 +240,11 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -29524,4 +29530,1282 @@
   <autoFilter ref="A19:J116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>AUTO EXPENSES BY COMPANY — fuel excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>De-duplicated: 5 Capital One rows ($2,127.99) that appear on two tabs each are counted once, under the entity their twin names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>COMPANY x CATEGORY  (both cards, de-duplicated)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
+      <c r="K4" s="5" t="n"/>
+      <c r="L4" s="5" t="n"/>
+      <c r="M4" s="5" t="n"/>
+      <c r="N4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Company / entity</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Charges</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Towing</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Car rental</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>Total $</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>58</v>
+      </c>
+      <c r="C6" s="54" t="n"/>
+      <c r="D6" s="54" t="n">
+        <v>3270.41</v>
+      </c>
+      <c r="E6" s="54" t="n">
+        <v>1410.22</v>
+      </c>
+      <c r="F6" s="54" t="n">
+        <v>1692.92</v>
+      </c>
+      <c r="G6" s="54" t="n">
+        <v>965.61</v>
+      </c>
+      <c r="H6" s="54" t="n"/>
+      <c r="I6" s="54" t="n">
+        <v>491.95</v>
+      </c>
+      <c r="J6" s="54" t="n"/>
+      <c r="K6" s="54" t="n">
+        <v>13</v>
+      </c>
+      <c r="L6" s="54" t="n">
+        <v>86.3</v>
+      </c>
+      <c r="M6" s="68" t="n">
+        <v>7930.41</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="54" t="n">
+        <v>3583.43</v>
+      </c>
+      <c r="D7" s="54" t="n"/>
+      <c r="E7" s="54" t="n"/>
+      <c r="F7" s="54" t="n"/>
+      <c r="G7" s="54" t="n"/>
+      <c r="H7" s="54" t="n">
+        <v>280</v>
+      </c>
+      <c r="I7" s="54" t="n"/>
+      <c r="J7" s="54" t="n"/>
+      <c r="K7" s="54" t="n"/>
+      <c r="L7" s="54" t="n"/>
+      <c r="M7" s="68" t="n">
+        <v>3863.43</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="52" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B8" s="52" t="n">
+        <v>25</v>
+      </c>
+      <c r="C8" s="53" t="n"/>
+      <c r="D8" s="53" t="n">
+        <v>700</v>
+      </c>
+      <c r="E8" s="53" t="n">
+        <v>1125.6</v>
+      </c>
+      <c r="F8" s="53" t="n"/>
+      <c r="G8" s="53" t="n"/>
+      <c r="H8" s="53" t="n"/>
+      <c r="I8" s="53" t="n"/>
+      <c r="J8" s="53" t="n">
+        <v>474.14</v>
+      </c>
+      <c r="K8" s="53" t="n">
+        <v>186</v>
+      </c>
+      <c r="L8" s="53" t="n">
+        <v>93.55</v>
+      </c>
+      <c r="M8" s="69" t="n">
+        <v>2579.29</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="54" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D9" s="54" t="n">
+        <v>263.5</v>
+      </c>
+      <c r="E9" s="54" t="n"/>
+      <c r="F9" s="54" t="n"/>
+      <c r="G9" s="54" t="n"/>
+      <c r="H9" s="54" t="n"/>
+      <c r="I9" s="54" t="n"/>
+      <c r="J9" s="54" t="n"/>
+      <c r="K9" s="54" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="L9" s="54" t="n"/>
+      <c r="M9" s="68" t="n">
+        <v>1474.29</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="55" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B10" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="56" t="n"/>
+      <c r="D10" s="56" t="n"/>
+      <c r="E10" s="56" t="n"/>
+      <c r="F10" s="56" t="n">
+        <v>12.95</v>
+      </c>
+      <c r="G10" s="56" t="n"/>
+      <c r="H10" s="56" t="n">
+        <v>400</v>
+      </c>
+      <c r="I10" s="56" t="n"/>
+      <c r="J10" s="56" t="n"/>
+      <c r="K10" s="56" t="n"/>
+      <c r="L10" s="56" t="n"/>
+      <c r="M10" s="43" t="n">
+        <v>412.95</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="65" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B11" s="66" t="n">
+        <v>92</v>
+      </c>
+      <c r="C11" s="44" t="n">
+        <v>4783.43</v>
+      </c>
+      <c r="D11" s="44" t="n">
+        <v>4233.91</v>
+      </c>
+      <c r="E11" s="44" t="n">
+        <v>2535.82</v>
+      </c>
+      <c r="F11" s="44" t="n">
+        <v>1705.87</v>
+      </c>
+      <c r="G11" s="44" t="n">
+        <v>965.61</v>
+      </c>
+      <c r="H11" s="44" t="n">
+        <v>680</v>
+      </c>
+      <c r="I11" s="44" t="n">
+        <v>491.95</v>
+      </c>
+      <c r="J11" s="44" t="n">
+        <v>474.14</v>
+      </c>
+      <c r="K11" s="44" t="n">
+        <v>209.79</v>
+      </c>
+      <c r="L11" s="44" t="n">
+        <v>179.85</v>
+      </c>
+      <c r="M11" s="67" t="n">
+        <v>16260.37</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>SPLIT BY CARD</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Company / entity</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Charges</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>AmEx $</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Capital One $</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Total $</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>58</v>
+      </c>
+      <c r="C15" s="54" t="n">
+        <v>6922.46</v>
+      </c>
+      <c r="D15" s="54" t="n">
+        <v>1007.95</v>
+      </c>
+      <c r="E15" s="54" t="n">
+        <v>7930.41</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>FasTrak $3,270 and tyres $1,693 dominate; no vehicle named on any toll</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="54" t="n">
+        <v>3583.43</v>
+      </c>
+      <c r="D16" s="54" t="n">
+        <v>280</v>
+      </c>
+      <c r="E16" s="54" t="n">
+        <v>3863.43</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Truck upfit $3,583 (bed cover + air suspension) and the F350 tow</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="52" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B17" s="52" t="n">
+        <v>25</v>
+      </c>
+      <c r="C17" s="53" t="n">
+        <v>1499.64</v>
+      </c>
+      <c r="D17" s="53" t="n">
+        <v>1079.65</v>
+      </c>
+      <c r="E17" s="53" t="n">
+        <v>2579.29</v>
+      </c>
+      <c r="F17" s="52" t="inlineStr">
+        <is>
+          <t>Personal — already tagged as such, still paid on the business cards</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="54" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="D18" s="54" t="n">
+        <v>1463.5</v>
+      </c>
+      <c r="E18" s="54" t="n">
+        <v>1474.29</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Van wrap $1,200 and FasTrak $264</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="55" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B19" s="55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="56" t="n">
+        <v>400</v>
+      </c>
+      <c r="D19" s="56" t="n">
+        <v>12.95</v>
+      </c>
+      <c r="E19" s="56" t="n">
+        <v>412.95</v>
+      </c>
+      <c r="F19" s="55" t="inlineStr">
+        <is>
+          <t>No entity on the row and no twin to inherit from</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="66" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B20" s="66" t="n">
+        <v>92</v>
+      </c>
+      <c r="C20" s="70" t="n">
+        <v>12416.32</v>
+      </c>
+      <c r="D20" s="70" t="n">
+        <v>3844.05</v>
+      </c>
+      <c r="E20" s="70" t="n">
+        <v>16260.37</v>
+      </c>
+      <c r="F20" s="71" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>CAPITAL ONE AUTO EXPENSES — every row, by company  (this is where the $230 would have to live)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Company / entity</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Source tab</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="n">
+        <v>46059</v>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>SQ *GOLDEN STATE WRAPS</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F24" s="30" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G24" s="16" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="n">
+        <v>46170</v>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>FasTrak</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F25" s="30" t="n">
+        <v>263.5</v>
+      </c>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F9-BULK TOLL, NO VEHICLE NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing — subtotal</t>
+        </is>
+      </c>
+      <c r="B26" s="52" t="n"/>
+      <c r="C26" s="52" t="n"/>
+      <c r="D26" s="52" t="n"/>
+      <c r="E26" s="52" t="n"/>
+      <c r="F26" s="69" t="n">
+        <v>1463.5</v>
+      </c>
+      <c r="G26" s="52" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="n">
+        <v>46151</v>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>State of California DMV</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F27" s="30" t="n">
+        <v>1059</v>
+      </c>
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="n">
+        <v>46151</v>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>DMV Fee</t>
+        </is>
+      </c>
+      <c r="E28" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F28" s="30" t="n">
+        <v>20.65</v>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F7-PERSONAL (OWNER PAY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="72" t="inlineStr">
+        <is>
+          <t>Owner's Pay — subtotal</t>
+        </is>
+      </c>
+      <c r="B29" s="52" t="n"/>
+      <c r="C29" s="52" t="n"/>
+      <c r="D29" s="52" t="n"/>
+      <c r="E29" s="52" t="n"/>
+      <c r="F29" s="69" t="n">
+        <v>1079.65</v>
+      </c>
+      <c r="G29" s="52" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B30" s="29" t="n">
+        <v>46059</v>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>FASTRAK</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F30" s="30" t="n">
+        <v>580</v>
+      </c>
+      <c r="G30" s="16" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket); F9-BULK TOLL, NO VEHICLE NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="n">
+        <v>46062</v>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F31" s="30" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="G31" s="16" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B32" s="29" t="n">
+        <v>46064</v>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>MTA Meter</t>
+        </is>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F32" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="G32" s="16" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B33" s="29" t="n">
+        <v>46090</v>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F33" s="30" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>F8-MISCODED AS FUEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B34" s="29" t="n">
+        <v>46121</v>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F34" s="30" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="G34" s="16" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B35" s="29" t="n">
+        <v>46151</v>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F35" s="30" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="G35" s="16" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B36" s="29" t="n">
+        <v>46165</v>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F36" s="30" t="n">
+        <v>60</v>
+      </c>
+      <c r="G36" s="16" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B37" s="29" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F37" s="30" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="G37" s="16" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F38" s="30" t="n">
+        <v>60</v>
+      </c>
+      <c r="G38" s="16" t="inlineStr">
+        <is>
+          <t>F6-UNCATEGORISED (blank bucket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="72" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track — subtotal</t>
+        </is>
+      </c>
+      <c r="B39" s="52" t="n"/>
+      <c r="C39" s="52" t="n"/>
+      <c r="D39" s="52" t="n"/>
+      <c r="E39" s="52" t="n"/>
+      <c r="F39" s="69" t="n">
+        <v>1007.95</v>
+      </c>
+      <c r="G39" s="52" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>Towing</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>Loural Towing</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F40" s="30" t="n">
+        <v>280</v>
+      </c>
+      <c r="G40" s="16" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="72" t="inlineStr">
+        <is>
+          <t>Matrix Group One — subtotal</t>
+        </is>
+      </c>
+      <c r="B41" s="52" t="n"/>
+      <c r="C41" s="52" t="n"/>
+      <c r="D41" s="52" t="n"/>
+      <c r="E41" s="52" t="n"/>
+      <c r="F41" s="69" t="n">
+        <v>280</v>
+      </c>
+      <c r="G41" s="52" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B42" s="29" t="n">
+        <v>46156</v>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>Autozone</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>Capital One Business Property E</t>
+        </is>
+      </c>
+      <c r="F42" s="30" t="n">
+        <v>12.95</v>
+      </c>
+      <c r="G42" s="16" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="72" t="inlineStr">
+        <is>
+          <t>Unassigned — subtotal</t>
+        </is>
+      </c>
+      <c r="B43" s="52" t="n"/>
+      <c r="C43" s="52" t="n"/>
+      <c r="D43" s="52" t="n"/>
+      <c r="E43" s="52" t="n"/>
+      <c r="F43" s="69" t="n">
+        <v>12.95</v>
+      </c>
+      <c r="G43" s="52" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="65" t="inlineStr">
+        <is>
+          <t>CAPITAL ONE AUTO TOTAL (de-duplicated)</t>
+        </is>
+      </c>
+      <c r="B44" s="71" t="n"/>
+      <c r="C44" s="71" t="n"/>
+      <c r="D44" s="71" t="n"/>
+      <c r="E44" s="71" t="n"/>
+      <c r="F44" s="67" t="n">
+        <v>3844.05</v>
+      </c>
+      <c r="G44" s="71" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>WHERE IS CAPITAL ONE'S $230?</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n"/>
+      <c r="C46" s="5" t="n"/>
+      <c r="D46" s="5" t="n"/>
+      <c r="E46" s="5" t="n"/>
+      <c r="F46" s="5" t="n"/>
+      <c r="G46" s="5" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>vs $230</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Tracker Vehicle/Field bucket — Real Estate entity</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>The tracker's own auto category for the main entity</t>
+        </is>
+      </c>
+      <c r="C48" s="54" t="n">
+        <v>127.98</v>
+      </c>
+      <c r="D48" s="54" t="n">
+        <v>-102.02</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Tracker Vehicle/Field bucket — all entities</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Adds Peninsula Plumbing and Matrix Group One</t>
+        </is>
+      </c>
+      <c r="C49" s="54" t="n">
+        <v>1990.03</v>
+      </c>
+      <c r="D49" s="54" t="n">
+        <v>1760.03</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>This audit — Cap One auto, Real Estate entity</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>De-duplicated, fuel excluded</t>
+        </is>
+      </c>
+      <c r="C50" s="54" t="n">
+        <v>1007.95</v>
+      </c>
+      <c r="D50" s="54" t="n">
+        <v>777.95</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>This audit — Cap One auto, all entities</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>De-duplicated, fuel excluded</t>
+        </is>
+      </c>
+      <c r="C51" s="54" t="n">
+        <v>3844.05</v>
+      </c>
+      <c r="D51" s="54" t="n">
+        <v>3614.05</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Closest single line: Loural Towing, Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Drop off Ford F350, 17-Feb-26</t>
+        </is>
+      </c>
+      <c r="C52" s="54" t="n">
+        <v>280</v>
+      </c>
+      <c r="D52" s="54" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="54" ht="32" customHeight="1">
+      <c r="A54" s="60" t="inlineStr">
+        <is>
+          <t>•  No cell in either workbook contains the value 230, and none contains 5,882.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="60" t="inlineStr">
+        <is>
+          <t>•  No company subtotal, category subtotal, month subtotal or bucket subtotal on the Capital One card equals $230.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="A56" s="60" t="inlineStr">
+        <is>
+          <t>•  An exhaustive search of every 1-, 2-, 3- and 4-row combination of Capital One fuel &amp; auto charges returns only coincidental sums — mixed dates, mixed categories, no coherent grouping. None is a real total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="32" customHeight="1">
+      <c r="A57" s="60" t="inlineStr">
+        <is>
+          <t>•  Conclusion: the $230 was not produced from the Capital One Expense Tracker as supplied. It comes from another source or an earlier snapshot. The nearest defensible figure for Capital One auto is $1,007.95 for the Real Estate entity, or $3,844.05 across all entities.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="A56:G56"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Capital One overhead-only fuel & auto tab
Rescopes to the four Capital One overhead tabs, excluding all property
tabs, per the tile's placement of Fuel & Auto under Overhead. Groups the
29 de-duplicated charges ($5,189.13) by entity with fuel and auto split
out and every row listed.

Records that the tile cannot be reproduced from these workbooks: no
Capital One subtotal equals $230, none equals the $6,629 Other Overhead
anchor, and the tile reports Capital One Software/Systems as nil while
the tracker carries $1,959.48 of it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X9qK8zkdfoo6K5q1ScTX2U
</commit_message>
<xml_diff>
--- a/audit/Fuel_Auto_Fraud_Audit.xlsx
+++ b/audit/Fuel_Auto_Fraud_Audit.xlsx
@@ -15,6 +15,7 @@
     <sheet name="6. Reconciliation" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="7. Auto Expenses Only" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="8. Auto by Company" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="9. Cap One Overhead F&amp;A" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Flagged Transactions'!$A$1:$N$175</definedName>
@@ -165,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -245,6 +246,8 @@
     <xf numFmtId="164" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -30808,4 +30811,1466 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F81"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>CAPITAL ONE — FUEL &amp; AUTO UNDER OVERHEAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Scope: the four overhead tabs only — Overhead Expenses, Personal Overhead Expenses, Business - Overhead Expense, PPS Expenses. All property tabs excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="38" t="inlineStr">
+        <is>
+          <t>De-duplicated: 7 rows ($2,296.16) appear on two tabs each and are counted once, under the entity their twin names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>FUEL &amp; AUTO UNDER OVERHEAD — BY COMPANY</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Company / entity</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Charges</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Fuel $</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Auto $</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Total $</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>15</v>
+      </c>
+      <c r="C7" s="54" t="n">
+        <v>1181.69</v>
+      </c>
+      <c r="D7" s="54" t="n">
+        <v>1463.5</v>
+      </c>
+      <c r="E7" s="68" t="n">
+        <v>2645.19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="52" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B8" s="52" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="53" t="n">
+        <v>78.68000000000001</v>
+      </c>
+      <c r="D8" s="53" t="n">
+        <v>1079.65</v>
+      </c>
+      <c r="E8" s="69" t="n">
+        <v>1158.33</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="54" t="n">
+        <v>97.66</v>
+      </c>
+      <c r="D9" s="54" t="n">
+        <v>1007.95</v>
+      </c>
+      <c r="E9" s="68" t="n">
+        <v>1105.61</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="54" t="n">
+        <v>280</v>
+      </c>
+      <c r="E10" s="68" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="65" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B11" s="66" t="n">
+        <v>29</v>
+      </c>
+      <c r="C11" s="67" t="n">
+        <v>1358.03</v>
+      </c>
+      <c r="D11" s="67" t="n">
+        <v>3831.1</v>
+      </c>
+      <c r="E11" s="67" t="n">
+        <v>5189.13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>AUTO EXPENSES UNDER OVERHEAD — every row</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Company / entity</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Description as booked</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Source tab</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="n">
+        <v>46059</v>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>SQ *GOLDEN STATE WRAPS</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>PPS - Van Wrap payment</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F15" s="30" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="n">
+        <v>46170</v>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>FasTrak</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr"/>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F16" s="30" t="n">
+        <v>263.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="72" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing — subtotal</t>
+        </is>
+      </c>
+      <c r="B17" s="52" t="n"/>
+      <c r="C17" s="52" t="n"/>
+      <c r="D17" s="52" t="n"/>
+      <c r="E17" s="52" t="n"/>
+      <c r="F17" s="69" t="n">
+        <v>1463.5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="n">
+        <v>46151</v>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>State of California DMV</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr"/>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="n">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="n">
+        <v>46151</v>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>DMV Fee</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr"/>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F19" s="30" t="n">
+        <v>20.65</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="72" t="inlineStr">
+        <is>
+          <t>Owner's Pay — subtotal</t>
+        </is>
+      </c>
+      <c r="B20" s="52" t="n"/>
+      <c r="C20" s="52" t="n"/>
+      <c r="D20" s="52" t="n"/>
+      <c r="E20" s="52" t="n"/>
+      <c r="F20" s="69" t="n">
+        <v>1079.65</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="n">
+        <v>46059</v>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>FASTRAK</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>FASTRAK</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F21" s="30" t="n">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="n">
+        <v>46062</v>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash Subscription</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F22" s="30" t="n">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B23" s="29" t="n">
+        <v>46064</v>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>MTA Meter</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>MTA Parking Meter Fee</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F23" s="30" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="n">
+        <v>46090</v>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr"/>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F24" s="30" t="n">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="n">
+        <v>46121</v>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr"/>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F25" s="30" t="n">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="n">
+        <v>46151</v>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr"/>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F26" s="30" t="n">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B27" s="29" t="n">
+        <v>46165</v>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F27" s="30" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr"/>
+      <c r="E28" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F28" s="30" t="n">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B29" s="29" t="n">
+        <v>46195</v>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr"/>
+      <c r="E29" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F29" s="30" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="72" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track — subtotal</t>
+        </is>
+      </c>
+      <c r="B30" s="52" t="n"/>
+      <c r="C30" s="52" t="n"/>
+      <c r="D30" s="52" t="n"/>
+      <c r="E30" s="52" t="n"/>
+      <c r="F30" s="69" t="n">
+        <v>1007.95</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Loural Towing</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Drop off Ford F350</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F31" s="30" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="72" t="inlineStr">
+        <is>
+          <t>Matrix Group One — subtotal</t>
+        </is>
+      </c>
+      <c r="B32" s="52" t="n"/>
+      <c r="C32" s="52" t="n"/>
+      <c r="D32" s="52" t="n"/>
+      <c r="E32" s="52" t="n"/>
+      <c r="F32" s="69" t="n">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="65" t="inlineStr">
+        <is>
+          <t>TOTAL AUTO</t>
+        </is>
+      </c>
+      <c r="B33" s="71" t="n"/>
+      <c r="C33" s="71" t="n"/>
+      <c r="D33" s="71" t="n"/>
+      <c r="E33" s="71" t="n"/>
+      <c r="F33" s="67" t="n">
+        <v>3831.1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>FUEL UNDER OVERHEAD — every row</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n"/>
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Company / entity</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Description as booked</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Source tab</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B37" s="29" t="n">
+        <v>46058</v>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>A&amp;A GAS AND FOOD MART</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Fuel for 2025 Ram Promaster 41406J4</t>
+        </is>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F37" s="30" t="n">
+        <v>82.66</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="n">
+        <v>46058</v>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>A&amp;A GAS AND FOOD MART</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>Fuel for 2025 Ram  41390J4</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F38" s="30" t="n">
+        <v>85.51000000000001</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="n">
+        <v>46086</v>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>Fuel for RAM 41406J4</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F39" s="30" t="n">
+        <v>115.88</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="n">
+        <v>46090</v>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>Chevron</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>Fuel for RAM 41406J4</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F40" s="30" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B41" s="29" t="n">
+        <v>46116</v>
+      </c>
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>A&amp;A GAS AND FOOD MART</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr"/>
+      <c r="E41" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F41" s="30" t="n">
+        <v>105.77</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B42" s="29" t="n">
+        <v>46132</v>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>ARCO</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr"/>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F42" s="30" t="n">
+        <v>121.86</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B43" s="29" t="n">
+        <v>46132</v>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>A&amp;A GAS AND FOOD MART</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr"/>
+      <c r="E43" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F43" s="30" t="n">
+        <v>109.8</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B44" s="29" t="n">
+        <v>46141</v>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>ARCO</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr"/>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F44" s="30" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B45" s="29" t="n">
+        <v>46150</v>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>A&amp;A GAS AND FOOD MART</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr"/>
+      <c r="E45" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F45" s="30" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B46" s="29" t="n">
+        <v>46157</v>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>ARCO $172.57</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr"/>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F46" s="30" t="n">
+        <v>57.52</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B47" s="29" t="n">
+        <v>46163</v>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>76 - $173.42</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr"/>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F47" s="30" t="n">
+        <v>36.48</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B48" s="29" t="n">
+        <v>46168</v>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>ARCO</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr"/>
+      <c r="E48" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F48" s="30" t="n">
+        <v>18.21</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B49" s="29" t="n">
+        <v>46186</v>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>ARCO</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>ARCO</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F49" s="30" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="72" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing — subtotal</t>
+        </is>
+      </c>
+      <c r="B50" s="52" t="n"/>
+      <c r="C50" s="52" t="n"/>
+      <c r="D50" s="52" t="n"/>
+      <c r="E50" s="52" t="n"/>
+      <c r="F50" s="69" t="n">
+        <v>1181.69</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B51" s="29" t="n">
+        <v>46142</v>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>Shell Oil</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr"/>
+      <c r="E51" s="16" t="inlineStr">
+        <is>
+          <t>Business - Overhead Expense</t>
+        </is>
+      </c>
+      <c r="F51" s="30" t="n">
+        <v>78.68000000000001</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="72" t="inlineStr">
+        <is>
+          <t>Owner's Pay — subtotal</t>
+        </is>
+      </c>
+      <c r="B52" s="52" t="n"/>
+      <c r="C52" s="52" t="n"/>
+      <c r="D52" s="52" t="n"/>
+      <c r="E52" s="52" t="n"/>
+      <c r="F52" s="69" t="n">
+        <v>78.68000000000001</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B53" s="29" t="n">
+        <v>46077</v>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>A&amp;A Gas and Food  Mart</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr"/>
+      <c r="E53" s="16" t="inlineStr">
+        <is>
+          <t>Personal Overhead Expenses</t>
+        </is>
+      </c>
+      <c r="F53" s="30" t="n">
+        <v>97.66</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="72" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track — subtotal</t>
+        </is>
+      </c>
+      <c r="B54" s="52" t="n"/>
+      <c r="C54" s="52" t="n"/>
+      <c r="D54" s="52" t="n"/>
+      <c r="E54" s="52" t="n"/>
+      <c r="F54" s="69" t="n">
+        <v>97.66</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="65" t="inlineStr">
+        <is>
+          <t>TOTAL FUEL</t>
+        </is>
+      </c>
+      <c r="B55" s="71" t="n"/>
+      <c r="C55" s="71" t="n"/>
+      <c r="D55" s="71" t="n"/>
+      <c r="E55" s="71" t="n"/>
+      <c r="F55" s="67" t="n">
+        <v>1358.03</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>THE $230 — EVERY CANDIDATE TESTED</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n"/>
+      <c r="C57" s="5" t="n"/>
+      <c r="D57" s="5" t="n"/>
+      <c r="E57" s="5" t="n"/>
+      <c r="F57" s="5" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>vs $230</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="55" t="inlineStr">
+        <is>
+          <t>Tracker's own Vehicle/Field bucket — Real Estate</t>
+        </is>
+      </c>
+      <c r="B59" s="55" t="inlineStr">
+        <is>
+          <t>The only auto category the tracker has, main entity</t>
+        </is>
+      </c>
+      <c r="C59" s="56" t="n">
+        <v>127.98</v>
+      </c>
+      <c r="D59" s="56" t="n">
+        <v>-102.02</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="55" t="inlineStr">
+        <is>
+          <t>Tracker's own Vehicle/Field bucket — all entities</t>
+        </is>
+      </c>
+      <c r="B60" s="55" t="inlineStr">
+        <is>
+          <t>Adds Peninsula Plumbing and Matrix Group One</t>
+        </is>
+      </c>
+      <c r="C60" s="56" t="n">
+        <v>1990.03</v>
+      </c>
+      <c r="D60" s="56" t="n">
+        <v>1760.03</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="55" t="inlineStr">
+        <is>
+          <t>This audit — auto under overhead, Real Estate</t>
+        </is>
+      </c>
+      <c r="B61" s="55" t="inlineStr">
+        <is>
+          <t>De-duplicated, fuel excluded</t>
+        </is>
+      </c>
+      <c r="C61" s="56" t="n">
+        <v>1007.95</v>
+      </c>
+      <c r="D61" s="56" t="n">
+        <v>777.95</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="55" t="inlineStr">
+        <is>
+          <t>This audit — auto under overhead, all entities</t>
+        </is>
+      </c>
+      <c r="B62" s="55" t="inlineStr">
+        <is>
+          <t>De-duplicated, fuel excluded</t>
+        </is>
+      </c>
+      <c r="C62" s="56" t="n">
+        <v>3831.1</v>
+      </c>
+      <c r="D62" s="56" t="n">
+        <v>3601.1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="55" t="inlineStr">
+        <is>
+          <t>This audit — fuel + auto under overhead, all entities</t>
+        </is>
+      </c>
+      <c r="B63" s="55" t="inlineStr">
+        <is>
+          <t>De-duplicated</t>
+        </is>
+      </c>
+      <c r="C63" s="56" t="n">
+        <v>5189.13</v>
+      </c>
+      <c r="D63" s="56" t="n">
+        <v>4959.13</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="55" t="inlineStr">
+        <is>
+          <t>Closest single line: Loural Towing (Matrix Group One)</t>
+        </is>
+      </c>
+      <c r="B64" s="55" t="inlineStr">
+        <is>
+          <t>Drop off Ford F350, 17-Feb-26</t>
+        </is>
+      </c>
+      <c r="C64" s="56" t="n">
+        <v>280</v>
+      </c>
+      <c r="D64" s="56" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>PROOF THE TILE WAS NOT BUILT FROM THIS WORKBOOK</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="n"/>
+      <c r="C66" s="5" t="n"/>
+      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="5" t="n"/>
+      <c r="F66" s="5" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="73" t="inlineStr">
+        <is>
+          <t>The tile shows a dash for Capital One Software/Systems — i.e. nothing. The tracker has $1,959.48 of it:</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="52" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B69" s="52" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+      <c r="C69" s="52" t="inlineStr">
+        <is>
+          <t>All Department - email and collaboration</t>
+        </is>
+      </c>
+      <c r="D69" s="53" t="n">
+        <v>871.48</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="52" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B70" s="52" t="inlineStr">
+        <is>
+          <t>Google Voice</t>
+        </is>
+      </c>
+      <c r="C70" s="52" t="inlineStr">
+        <is>
+          <t>Google Voice for all Employees</t>
+        </is>
+      </c>
+      <c r="D70" s="53" t="n">
+        <v>743.2</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="52" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B71" s="52" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="C71" s="52" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="D71" s="53" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="52" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="B72" s="52" t="inlineStr">
+        <is>
+          <t>Intuit</t>
+        </is>
+      </c>
+      <c r="C72" s="52" t="inlineStr">
+        <is>
+          <t>Intuit</t>
+        </is>
+      </c>
+      <c r="D72" s="53" t="n">
+        <v>44.8</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="55" t="n"/>
+      <c r="B73" s="55" t="n"/>
+      <c r="C73" s="46" t="inlineStr">
+        <is>
+          <t>TOTAL — reported as "—" on the tile</t>
+        </is>
+      </c>
+      <c r="D73" s="74" t="n">
+        <v>1959.48</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="59" t="inlineStr">
+        <is>
+          <t>FINDINGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="46" customHeight="1">
+      <c r="A76" s="60" t="inlineStr">
+        <is>
+          <t>•  There is no category called "Auto Expense" anywhere in the Capital One tracker. The tracker's only auto grouping is the Bucket column value "Vehicle/Field", and that column is populated on exactly one tab — Personal Overhead Expenses. On the other three overhead tabs the Bucket column is entirely blank, so those charges belong to no category at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="46" customHeight="1">
+      <c r="A77" s="60" t="inlineStr">
+        <is>
+          <t>•  Restricted to overhead as you describe it, Capital One fuel &amp; auto is $5,189.13 de-duplicated — $1,358.03 of fuel and $3,831.10 of auto. The tracker's own Vehicle/Field bucket captures only $1,990.03 of that; the remaining $3,199.10 sits in blank-bucket rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="46" customHeight="1">
+      <c r="A78" s="60" t="inlineStr">
+        <is>
+          <t>•  No subtotal in the Capital One overhead tabs equals $230 — not by company, category, bucket, month, or tab. No cell in the workbook contains the value 230.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="46" customHeight="1">
+      <c r="A79" s="60" t="inlineStr">
+        <is>
+          <t>•  The tile's other Capital One anchor fails the same test: "Other Overhead $6,629" matches no subtotal either. The closest is the Operations bucket at $6,621.53, which is $7.47 away and would pair with Fuel &amp; Auto of $1,990.03, not $230.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="46" customHeight="1">
+      <c r="A80" s="60" t="inlineStr">
+        <is>
+          <t>•  All three AmEx anchors fail too — no combination of rows, buckets, entities, months or cumulative periods produces $33,443, $17,245 or $5,882.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="46" customHeight="1">
+      <c r="A81" s="60" t="inlineStr">
+        <is>
+          <t>•  Conclusion: the category tile was not generated from these two workbooks. The Software/Systems dash proves it directly — the Capital One card plainly carries $1,959.48 of software, so a report showing nothing there is reading a different dataset.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A76:F76"/>
+    <mergeCell ref="A80:F80"/>
+    <mergeCell ref="A79:F79"/>
+    <mergeCell ref="A78:F78"/>
+    <mergeCell ref="A77:F77"/>
+    <mergeCell ref="A81:F81"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add AmEx overhead-only fuel & auto tab with dashboard comparison
Rescopes AmEx to the overhead tab and groups the 151 charges
($16,925.87) by entity and category.

Records the decisive test: the AmEx workbook's own dashboard tab, on the
same company filter, reports Vehicle/Field at $6,148.72 across 51
transactions against the tile's $5,882. All three overhead rows are
short and the total is short by the same $2,646.49, which rules out a
category-definition difference.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X9qK8zkdfoo6K5q1ScTX2U
</commit_message>
<xml_diff>
--- a/audit/Fuel_Auto_Fraud_Audit.xlsx
+++ b/audit/Fuel_Auto_Fraud_Audit.xlsx
@@ -16,6 +16,7 @@
     <sheet name="7. Auto Expenses Only" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="8. Auto by Company" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="9. Cap One Overhead F&amp;A" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="10. AmEx Overhead F&amp;A" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Flagged Transactions'!$A$1:$N$175</definedName>
@@ -1353,6 +1354,3012 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L116"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>AMEX — FUEL &amp; AUTO UNDER OVERHEAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Scope: the AmEx overhead tab only (Copy of Overhead Expenses). Property Expenses excluded. The stale "Overhead Expenses" tab is excluded — 414 of its 421 rows are repeats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>THE ANSWER: THE WORKBOOK'S OWN DASHBOARD DISAGREES WITH THE TILE</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>The AmEx workbook has a built-in dashboard tab ("Overhead Expenses dashboard"), filtered to Company = Real Estate- THB/ Equity Track. Here is what it reports against your tile:</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Overhead row</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Your tile</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Workbook dashboard</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Dashboard cell</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Shortfall</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="55" t="inlineStr">
+        <is>
+          <t>Fuel &amp; Auto  (bucket: Vehicle/Field)</t>
+        </is>
+      </c>
+      <c r="B7" s="56" t="n">
+        <v>5882</v>
+      </c>
+      <c r="C7" s="56" t="n">
+        <v>6148.72</v>
+      </c>
+      <c r="D7" s="55" t="inlineStr">
+        <is>
+          <t>dashboard r14 c2</t>
+        </is>
+      </c>
+      <c r="E7" s="56" t="n">
+        <v>266.72</v>
+      </c>
+      <c r="F7" s="55" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="55" t="inlineStr">
+        <is>
+          <t>Software/Systems</t>
+        </is>
+      </c>
+      <c r="B8" s="56" t="n">
+        <v>17245</v>
+      </c>
+      <c r="C8" s="56" t="n">
+        <v>17828.5</v>
+      </c>
+      <c r="D8" s="55" t="inlineStr">
+        <is>
+          <t>dashboard r11 c2</t>
+        </is>
+      </c>
+      <c r="E8" s="56" t="n">
+        <v>583.5</v>
+      </c>
+      <c r="F8" s="55" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="55" t="inlineStr">
+        <is>
+          <t>Other Overhead  (bucket: No Category)</t>
+        </is>
+      </c>
+      <c r="B9" s="56" t="n">
+        <v>33443</v>
+      </c>
+      <c r="C9" s="56" t="n">
+        <v>35239.27</v>
+      </c>
+      <c r="D9" s="55" t="inlineStr">
+        <is>
+          <t>dashboard r18 c2</t>
+        </is>
+      </c>
+      <c r="E9" s="56" t="n">
+        <v>1796.27</v>
+      </c>
+      <c r="F9" s="55" t="n">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="65" t="inlineStr">
+        <is>
+          <t>TOTAL OVERHEAD</t>
+        </is>
+      </c>
+      <c r="B10" s="67" t="n">
+        <v>56570</v>
+      </c>
+      <c r="C10" s="67" t="n">
+        <v>59216.49</v>
+      </c>
+      <c r="D10" s="71" t="n"/>
+      <c r="E10" s="67" t="n">
+        <v>2646.49</v>
+      </c>
+      <c r="F10" s="71" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="38" t="inlineStr">
+        <is>
+          <t>Every row is short, and the total is short by the same $2,646.49. A category-definition difference would move money between rows and leave the total intact — so this is roughly $2,646 of transactions the tile never saw, not a classification disagreement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>AMEX FUEL &amp; AUTO UNDER OVERHEAD — BY COMPANY  (this audit)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Company / entity</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Charges</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Fuel $</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Auto $</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Total $</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Tracker Vehicle/Field bucket $</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>100</v>
+      </c>
+      <c r="C15" s="54" t="n">
+        <v>3361.13</v>
+      </c>
+      <c r="D15" s="54" t="n">
+        <v>6014.55</v>
+      </c>
+      <c r="E15" s="68" t="n">
+        <v>9375.68</v>
+      </c>
+      <c r="F15" s="54" t="n">
+        <v>6148.72</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="52" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B16" s="52" t="n">
+        <v>45</v>
+      </c>
+      <c r="C16" s="53" t="n">
+        <v>2262.76</v>
+      </c>
+      <c r="D16" s="53" t="n">
+        <v>1499.64</v>
+      </c>
+      <c r="E16" s="69" t="n">
+        <v>3762.4</v>
+      </c>
+      <c r="F16" s="53" t="n">
+        <v>879.42</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="54" t="n">
+        <v>3583.43</v>
+      </c>
+      <c r="E17" s="68" t="n">
+        <v>3583.43</v>
+      </c>
+      <c r="F17" s="54" t="n">
+        <v>3583.43</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="54" t="n">
+        <v>193.57</v>
+      </c>
+      <c r="D18" s="54" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="E18" s="68" t="n">
+        <v>204.36</v>
+      </c>
+      <c r="F18" s="54" t="n">
+        <v>204.36</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="65" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B19" s="66" t="n">
+        <v>151</v>
+      </c>
+      <c r="C19" s="67" t="n">
+        <v>5817.46</v>
+      </c>
+      <c r="D19" s="67" t="n">
+        <v>11108.41</v>
+      </c>
+      <c r="E19" s="67" t="n">
+        <v>16925.87</v>
+      </c>
+      <c r="F19" s="67" t="n">
+        <v>10815.93</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>BY COMPANY x CATEGORY</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Company / entity</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Fuel (pump/station)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Car rental</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>Total $</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B23" s="54" t="n">
+        <v>3361.13</v>
+      </c>
+      <c r="C23" s="54" t="n">
+        <v>1782.5</v>
+      </c>
+      <c r="D23" s="54" t="n">
+        <v>1692.92</v>
+      </c>
+      <c r="E23" s="54" t="n">
+        <v>1410.22</v>
+      </c>
+      <c r="F23" s="54" t="n">
+        <v>545.66</v>
+      </c>
+      <c r="G23" s="54" t="n">
+        <v>491.95</v>
+      </c>
+      <c r="H23" s="54" t="n"/>
+      <c r="I23" s="54" t="n">
+        <v>5</v>
+      </c>
+      <c r="J23" s="54" t="n">
+        <v>86.3</v>
+      </c>
+      <c r="K23" s="54" t="n"/>
+      <c r="L23" s="68" t="n">
+        <v>9375.68</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B24" s="54" t="n">
+        <v>2262.76</v>
+      </c>
+      <c r="C24" s="54" t="n">
+        <v>700</v>
+      </c>
+      <c r="D24" s="54" t="n"/>
+      <c r="E24" s="54" t="n">
+        <v>45.95</v>
+      </c>
+      <c r="F24" s="54" t="n"/>
+      <c r="G24" s="54" t="n"/>
+      <c r="H24" s="54" t="n">
+        <v>474.14</v>
+      </c>
+      <c r="I24" s="54" t="n">
+        <v>186</v>
+      </c>
+      <c r="J24" s="54" t="n">
+        <v>93.55</v>
+      </c>
+      <c r="K24" s="54" t="n"/>
+      <c r="L24" s="68" t="n">
+        <v>3762.4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B25" s="54" t="n"/>
+      <c r="C25" s="54" t="n"/>
+      <c r="D25" s="54" t="n"/>
+      <c r="E25" s="54" t="n"/>
+      <c r="F25" s="54" t="n"/>
+      <c r="G25" s="54" t="n"/>
+      <c r="H25" s="54" t="n"/>
+      <c r="I25" s="54" t="n"/>
+      <c r="J25" s="54" t="n"/>
+      <c r="K25" s="54" t="n">
+        <v>3583.43</v>
+      </c>
+      <c r="L25" s="68" t="n">
+        <v>3583.43</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B26" s="54" t="n">
+        <v>193.57</v>
+      </c>
+      <c r="C26" s="54" t="n"/>
+      <c r="D26" s="54" t="n"/>
+      <c r="E26" s="54" t="n"/>
+      <c r="F26" s="54" t="n"/>
+      <c r="G26" s="54" t="n"/>
+      <c r="H26" s="54" t="n"/>
+      <c r="I26" s="54" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="J26" s="54" t="n"/>
+      <c r="K26" s="54" t="n"/>
+      <c r="L26" s="68" t="n">
+        <v>204.36</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="66" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="44" t="n">
+        <v>5817.46</v>
+      </c>
+      <c r="C27" s="44" t="n">
+        <v>2482.5</v>
+      </c>
+      <c r="D27" s="44" t="n">
+        <v>1692.92</v>
+      </c>
+      <c r="E27" s="44" t="n">
+        <v>1456.17</v>
+      </c>
+      <c r="F27" s="44" t="n">
+        <v>545.66</v>
+      </c>
+      <c r="G27" s="44" t="n">
+        <v>491.95</v>
+      </c>
+      <c r="H27" s="44" t="n">
+        <v>474.14</v>
+      </c>
+      <c r="I27" s="44" t="n">
+        <v>201.79</v>
+      </c>
+      <c r="J27" s="44" t="n">
+        <v>179.85</v>
+      </c>
+      <c r="K27" s="44" t="n">
+        <v>3583.43</v>
+      </c>
+      <c r="L27" s="67" t="n">
+        <v>16925.87</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>AUTO EXPENSES UNDER OVERHEAD — every row (fuel listed on tab 3)</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Company / entity</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Description as booked</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Bucket as booked</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="n">
+        <v>45889</v>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track – SFO prepaid parking</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="G31" s="30" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B32" s="29" t="n">
+        <v>45893</v>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track – SFO prepaid parking</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="G32" s="30" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B33" s="29" t="n">
+        <v>45895</v>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>Bobcat of the Bay</t>
+        </is>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track – Bobcat supplies (hoses, couplers, hydraulic parts)</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G33" s="30" t="n">
+        <v>517.89</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B34" s="29" t="n">
+        <v>45897</v>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track – car wash expense</t>
+        </is>
+      </c>
+      <c r="F34" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G34" s="30" t="n">
+        <v>49.99</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B35" s="29" t="n">
+        <v>45941</v>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing (Auto Pride)</t>
+        </is>
+      </c>
+      <c r="F35" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G35" s="30" t="n">
+        <v>5.75</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B36" s="29" t="n">
+        <v>45944</v>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track – SFO prepaid parking</t>
+        </is>
+      </c>
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="G36" s="30" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B37" s="29" t="n">
+        <v>45944</v>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing</t>
+        </is>
+      </c>
+      <c r="F37" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G37" s="30" t="n">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="n">
+        <v>45945</v>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track – SFO prepaid parking</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="G38" s="30" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="n">
+        <v>45945</v>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – parking citation/fine Juan's Mercedes</t>
+        </is>
+      </c>
+      <c r="F39" s="16" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="G39" s="30" t="n">
+        <v>105.95</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="n">
+        <v>45958</v>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>Auto Expenses - Equity Track Inc</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G40" s="30" t="n">
+        <v>49.99</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B41" s="29" t="n">
+        <v>45974</v>
+      </c>
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>Beltran Tire Service</t>
+        </is>
+      </c>
+      <c r="E41" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – vehicle tire service/repair</t>
+        </is>
+      </c>
+      <c r="F41" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G41" s="30" t="n">
+        <v>1140.03</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B42" s="29" t="n">
+        <v>45975</v>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G42" s="30" t="n">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B43" s="29" t="n">
+        <v>45976</v>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>Parking Citation Service Center</t>
+        </is>
+      </c>
+      <c r="E43" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – airport parking/terminal expense (San Jose)</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="G43" s="30" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B44" s="29" t="n">
+        <v>45983</v>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G44" s="30" t="n">
+        <v>79.98999999999999</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B45" s="29" t="n">
+        <v>45989</v>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E45" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G45" s="30" t="n">
+        <v>49.99</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B46" s="29" t="n">
+        <v>45999</v>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>CA DMV</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – DMV vehicle filing/processing fee</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G46" s="30" t="n">
+        <v>10.18</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B47" s="29" t="n">
+        <v>45999</v>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>CA DMV</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – DMV vehicle registration/service fee</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G47" s="30" t="n">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B48" s="29" t="n">
+        <v>46005</v>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E48" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – car wash/auto detailing</t>
+        </is>
+      </c>
+      <c r="F48" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G48" s="30" t="n">
+        <v>59.99</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B49" s="29" t="n">
+        <v>46008</v>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>CA DMV</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle registration or DMV fee</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G49" s="30" t="n">
+        <v>17.04</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B50" s="29" t="n">
+        <v>46008</v>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>State of California</t>
+        </is>
+      </c>
+      <c r="E50" s="16" t="inlineStr">
+        <is>
+          <t>DMV payment (license/registration)</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G50" s="30" t="n">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B51" s="29" t="n">
+        <v>46013</v>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E51" s="16" t="inlineStr">
+        <is>
+          <t>Car wash</t>
+        </is>
+      </c>
+      <c r="F51" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G51" s="30" t="n">
+        <v>79.98999999999999</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B52" s="29" t="n">
+        <v>46019</v>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>Car wash / detailing</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>Auto Pride Car Wash</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="inlineStr">
+        <is>
+          <t>Car wash</t>
+        </is>
+      </c>
+      <c r="F52" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G52" s="30" t="n">
+        <v>49.99</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B53" s="29" t="n">
+        <v>46080</v>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>LAZ PARKING</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="inlineStr"/>
+      <c r="F53" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G53" s="30" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B54" s="29" t="n">
+        <v>46094</v>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>Citations / fines</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>SFMTA CIT PYMNT WEB</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr"/>
+      <c r="F54" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G54" s="30" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B55" s="29" t="n">
+        <v>46114</v>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>Fastrak</t>
+        </is>
+      </c>
+      <c r="E55" s="16" t="inlineStr"/>
+      <c r="F55" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G55" s="30" t="n">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B56" s="29" t="n">
+        <v>46128</v>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>FASTRAK VIOLATION CESAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="inlineStr"/>
+      <c r="F56" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G56" s="30" t="n">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B57" s="29" t="n">
+        <v>46131</v>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>FASTRAK CSC TOLLS OAKLAND CA</t>
+        </is>
+      </c>
+      <c r="E57" s="16" t="inlineStr"/>
+      <c r="F57" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G57" s="30" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B58" s="29" t="n">
+        <v>46166</v>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D58" s="16" t="inlineStr">
+        <is>
+          <t>FASTRAK VIOLATION CESAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr"/>
+      <c r="F58" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G58" s="30" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B59" s="29" t="n">
+        <v>46183</v>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E59" s="16" t="inlineStr"/>
+      <c r="F59" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G59" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B60" s="29" t="n">
+        <v>46183</v>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr"/>
+      <c r="F60" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G60" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B61" s="29" t="n">
+        <v>46184</v>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="inlineStr"/>
+      <c r="F61" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G61" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B62" s="29" t="n">
+        <v>46184</v>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr"/>
+      <c r="F62" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G62" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B63" s="29" t="n">
+        <v>46203</v>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER PHONESAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="inlineStr"/>
+      <c r="F63" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G63" s="30" t="n">
+        <v>-2.05</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B64" s="29" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr"/>
+      <c r="F64" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G64" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B65" s="29" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="inlineStr"/>
+      <c r="F65" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G65" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B66" s="29" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANC</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="inlineStr"/>
+      <c r="F66" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G66" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B67" s="29" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C67" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D67" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANC</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="inlineStr"/>
+      <c r="F67" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G67" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B68" s="29" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E68" s="16" t="inlineStr"/>
+      <c r="F68" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G68" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B69" s="29" t="n">
+        <v>46211</v>
+      </c>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="inlineStr"/>
+      <c r="F69" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G69" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B70" s="29" t="n">
+        <v>46213</v>
+      </c>
+      <c r="C70" s="16" t="inlineStr">
+        <is>
+          <t>Tires / parts / repairs</t>
+        </is>
+      </c>
+      <c r="D70" s="16" t="inlineStr">
+        <is>
+          <t>BELTRAN TIRES INC - REDWOOD CITY CA</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="inlineStr"/>
+      <c r="F70" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G70" s="30" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B71" s="29" t="n">
+        <v>46218</v>
+      </c>
+      <c r="C71" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D71" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="inlineStr"/>
+      <c r="F71" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G71" s="30" t="n">
+        <v>5.85</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B72" s="29" t="n">
+        <v>46219</v>
+      </c>
+      <c r="C72" s="16" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D72" s="16" t="inlineStr">
+        <is>
+          <t>FASTRAK</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="inlineStr"/>
+      <c r="F72" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G72" s="30" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B73" s="29" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
+        <is>
+          <t>Clipper Trans</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr"/>
+      <c r="F73" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G73" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B74" s="29" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C74" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D74" s="16" t="inlineStr">
+        <is>
+          <t>Clipper Trans</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr"/>
+      <c r="F74" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G74" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B75" s="29" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>Clipper Trans</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr"/>
+      <c r="F75" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G75" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B76" s="29" t="n">
+        <v>46226</v>
+      </c>
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>Clipper Trans</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr"/>
+      <c r="F76" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G76" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="16" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track</t>
+        </is>
+      </c>
+      <c r="B77" s="29" t="n">
+        <v>46228</v>
+      </c>
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>Clipper Trans</t>
+        </is>
+      </c>
+      <c r="E77" s="16" t="inlineStr"/>
+      <c r="F77" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G77" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="72" t="inlineStr">
+        <is>
+          <t>Real Estate- THB/ Equity Track — subtotal</t>
+        </is>
+      </c>
+      <c r="B78" s="52" t="n"/>
+      <c r="C78" s="52" t="n"/>
+      <c r="D78" s="52" t="n"/>
+      <c r="E78" s="52" t="n"/>
+      <c r="F78" s="52" t="n"/>
+      <c r="G78" s="69" t="n">
+        <v>6014.55</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B79" s="29" t="n">
+        <v>45894</v>
+      </c>
+      <c r="C79" s="16" t="inlineStr">
+        <is>
+          <t>Car rental</t>
+        </is>
+      </c>
+      <c r="D79" s="16" t="inlineStr">
+        <is>
+          <t>Enterprise Rent-A-Car</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>Travel – car rental (Mariaelena) - Equity Track</t>
+        </is>
+      </c>
+      <c r="F79" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G79" s="30" t="n">
+        <v>474.14</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B80" s="29" t="n">
+        <v>46014</v>
+      </c>
+      <c r="C80" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D80" s="16" t="inlineStr">
+        <is>
+          <t>CA DMV</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle registration or DMV fee - Lucas's DMV Schedule</t>
+        </is>
+      </c>
+      <c r="F80" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G80" s="30" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B81" s="29" t="n">
+        <v>46014</v>
+      </c>
+      <c r="C81" s="16" t="inlineStr">
+        <is>
+          <t>DMV / registration</t>
+        </is>
+      </c>
+      <c r="D81" s="16" t="inlineStr">
+        <is>
+          <t>CA DMV</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle registration or DMV fee - Lucas's DMV Schedule</t>
+        </is>
+      </c>
+      <c r="F81" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G81" s="30" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B82" s="29" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D82" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr"/>
+      <c r="F82" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G82" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B83" s="29" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C83" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D83" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E83" s="16" t="inlineStr"/>
+      <c r="F83" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G83" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B84" s="29" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C84" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D84" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E84" s="16" t="inlineStr"/>
+      <c r="F84" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G84" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B85" s="29" t="n">
+        <v>46177</v>
+      </c>
+      <c r="C85" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D85" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E85" s="16" t="inlineStr"/>
+      <c r="F85" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G85" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B86" s="29" t="n">
+        <v>46178</v>
+      </c>
+      <c r="C86" s="16" t="inlineStr">
+        <is>
+          <t>Tolls (FasTrak)</t>
+        </is>
+      </c>
+      <c r="D86" s="16" t="inlineStr">
+        <is>
+          <t>FASTRAK CSC TOLLS</t>
+        </is>
+      </c>
+      <c r="E86" s="16" t="inlineStr"/>
+      <c r="F86" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G86" s="30" t="n">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B87" s="29" t="n">
+        <v>46178</v>
+      </c>
+      <c r="C87" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E87" s="16" t="inlineStr"/>
+      <c r="F87" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G87" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B88" s="29" t="n">
+        <v>46178</v>
+      </c>
+      <c r="C88" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D88" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr"/>
+      <c r="F88" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G88" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B89" s="29" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C89" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D89" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="inlineStr"/>
+      <c r="F89" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G89" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B90" s="29" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C90" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="inlineStr"/>
+      <c r="F90" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G90" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B91" s="29" t="n">
+        <v>46183</v>
+      </c>
+      <c r="C91" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E91" s="16" t="inlineStr"/>
+      <c r="F91" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G91" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B92" s="29" t="n">
+        <v>46189</v>
+      </c>
+      <c r="C92" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D92" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E92" s="16" t="inlineStr"/>
+      <c r="F92" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G92" s="30" t="n">
+        <v>2.05</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B93" s="29" t="n">
+        <v>46198</v>
+      </c>
+      <c r="C93" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E93" s="16" t="inlineStr"/>
+      <c r="F93" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G93" s="30" t="n">
+        <v>7.55</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B94" s="29" t="n">
+        <v>46198</v>
+      </c>
+      <c r="C94" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D94" s="16" t="inlineStr">
+        <is>
+          <t>CLIPPER-TRANSIT FARE</t>
+        </is>
+      </c>
+      <c r="E94" s="16" t="inlineStr"/>
+      <c r="F94" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G94" s="30" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B95" s="29" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C95" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E95" s="16" t="inlineStr"/>
+      <c r="F95" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G95" s="30" t="n">
+        <v>7.55</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B96" s="29" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C96" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D96" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E96" s="16" t="inlineStr"/>
+      <c r="F96" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G96" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B97" s="29" t="n">
+        <v>46209</v>
+      </c>
+      <c r="C97" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D97" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E97" s="16" t="inlineStr"/>
+      <c r="F97" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G97" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B98" s="29" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C98" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D98" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO       CA</t>
+        </is>
+      </c>
+      <c r="E98" s="16" t="inlineStr"/>
+      <c r="F98" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G98" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B99" s="29" t="n">
+        <v>46210</v>
+      </c>
+      <c r="C99" s="16" t="inlineStr">
+        <is>
+          <t>Transit (Clipper)</t>
+        </is>
+      </c>
+      <c r="D99" s="16" t="inlineStr">
+        <is>
+          <t>AplPay CLIPPER TRANSSAN FRANCISCO       CA</t>
+        </is>
+      </c>
+      <c r="E99" s="16" t="inlineStr"/>
+      <c r="F99" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G99" s="30" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B100" s="29" t="n">
+        <v>46217</v>
+      </c>
+      <c r="C100" s="16" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D100" s="16" t="inlineStr">
+        <is>
+          <t>82858 - TERMINAL A ESAN JOSE CA</t>
+        </is>
+      </c>
+      <c r="E100" s="16" t="inlineStr"/>
+      <c r="F100" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G100" s="30" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="16" t="inlineStr">
+        <is>
+          <t>Owner's Pay</t>
+        </is>
+      </c>
+      <c r="B101" s="29" t="n">
+        <v>46217</v>
+      </c>
+      <c r="C101" s="16" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D101" s="16" t="inlineStr">
+        <is>
+          <t>60774 - SFO PARKING SAN FRANCISCO CA</t>
+        </is>
+      </c>
+      <c r="E101" s="16" t="inlineStr"/>
+      <c r="F101" s="22" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="G101" s="30" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="72" t="inlineStr">
+        <is>
+          <t>Owner's Pay — subtotal</t>
+        </is>
+      </c>
+      <c r="B102" s="52" t="n"/>
+      <c r="C102" s="52" t="n"/>
+      <c r="D102" s="52" t="n"/>
+      <c r="E102" s="52" t="n"/>
+      <c r="F102" s="52" t="n"/>
+      <c r="G102" s="69" t="n">
+        <v>1499.64</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="16" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B103" s="29" t="n">
+        <v>45975</v>
+      </c>
+      <c r="C103" s="16" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="D103" s="16" t="inlineStr">
+        <is>
+          <t>BTPeragon Enterprises</t>
+        </is>
+      </c>
+      <c r="E103" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – truck bed cover (BTperagon)</t>
+        </is>
+      </c>
+      <c r="F103" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G103" s="30" t="n">
+        <v>1530.16</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="16" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B104" s="29" t="n">
+        <v>45975</v>
+      </c>
+      <c r="C104" s="16" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="D104" s="16" t="inlineStr">
+        <is>
+          <t>Logiq Air Suspension Solutions</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – air suspension remote (Logiq Air system)</t>
+        </is>
+      </c>
+      <c r="F104" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G104" s="30" t="n">
+        <v>174.01</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="16" t="inlineStr">
+        <is>
+          <t>Matrix Group One</t>
+        </is>
+      </c>
+      <c r="B105" s="29" t="n">
+        <v>45975</v>
+      </c>
+      <c r="C105" s="16" t="inlineStr">
+        <is>
+          <t>Truck upfit / equipment</t>
+        </is>
+      </c>
+      <c r="D105" s="16" t="inlineStr">
+        <is>
+          <t>Logiq Air Suspension Solutions</t>
+        </is>
+      </c>
+      <c r="E105" s="16" t="inlineStr">
+        <is>
+          <t>Equity Track Inc – truck air suspension kit (Logiq Air)</t>
+        </is>
+      </c>
+      <c r="F105" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G105" s="30" t="n">
+        <v>1879.26</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="72" t="inlineStr">
+        <is>
+          <t>Matrix Group One — subtotal</t>
+        </is>
+      </c>
+      <c r="B106" s="52" t="n"/>
+      <c r="C106" s="52" t="n"/>
+      <c r="D106" s="52" t="n"/>
+      <c r="E106" s="52" t="n"/>
+      <c r="F106" s="52" t="n"/>
+      <c r="G106" s="69" t="n">
+        <v>3583.43</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="16" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing</t>
+        </is>
+      </c>
+      <c r="B107" s="29" t="n">
+        <v>46100</v>
+      </c>
+      <c r="C107" s="16" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="D107" s="16" t="inlineStr">
+        <is>
+          <t>MTA METERS - MTA PBP</t>
+        </is>
+      </c>
+      <c r="E107" s="16" t="inlineStr">
+        <is>
+          <t>Parking Payment for Alan</t>
+        </is>
+      </c>
+      <c r="F107" s="16" t="inlineStr">
+        <is>
+          <t>Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="G107" s="30" t="n">
+        <v>10.79</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="72" t="inlineStr">
+        <is>
+          <t>Peninsula Plumbing — subtotal</t>
+        </is>
+      </c>
+      <c r="B108" s="52" t="n"/>
+      <c r="C108" s="52" t="n"/>
+      <c r="D108" s="52" t="n"/>
+      <c r="E108" s="52" t="n"/>
+      <c r="F108" s="52" t="n"/>
+      <c r="G108" s="69" t="n">
+        <v>10.79</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="65" t="inlineStr">
+        <is>
+          <t>TOTAL AUTO UNDER OVERHEAD</t>
+        </is>
+      </c>
+      <c r="B109" s="71" t="n"/>
+      <c r="C109" s="71" t="n"/>
+      <c r="D109" s="71" t="n"/>
+      <c r="E109" s="71" t="n"/>
+      <c r="F109" s="71" t="n"/>
+      <c r="G109" s="67" t="n">
+        <v>11108.41</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="59" t="inlineStr">
+        <is>
+          <t>WHY $5,882 CANNOT BE PRODUCED FROM THIS WORKBOOK</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="46" customHeight="1">
+      <c r="A112" s="60" t="inlineStr">
+        <is>
+          <t>•  The workbook's own dashboard, on the same Company filter, reports Vehicle/Field at $6,148.72 across 51 transactions. The tile says $5,882. The workbook disagrees with the tile by $266.72.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="46" customHeight="1">
+      <c r="A113" s="60" t="inlineStr">
+        <is>
+          <t>•  Every combination was tested and none produces $5,882: every bucket, every entity subset, every expense-type subset, every contiguous month window, every cumulative period, and every combination of those. Searches within $2 of the target return only arbitrary mixtures — drop DMV, Parking and Tolls but keep the rest, over Oct-2025 to May-2026 — which are search artifacts, not a definition anyone would report on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="46" customHeight="1">
+      <c r="A114" s="60" t="inlineStr">
+        <is>
+          <t>•  The "earlier snapshot" theory was tested too: if the tile predated some entries, the shortfall would equal the most recent rows in each bucket. It does not, in any of the three buckets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="46" customHeight="1">
+      <c r="A115" s="60" t="inlineStr">
+        <is>
+          <t>•  The shortfall is consistent across all three overhead rows and the total is short by exactly the same $2,646.49. That rules out a category-definition difference, which would shuffle money between rows while preserving the total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="46" customHeight="1">
+      <c r="A116" s="60" t="inlineStr">
+        <is>
+          <t>•  The real figure for AmEx fuel &amp; auto under overhead is $16,925.87 across 151 charges, of which the tracker's Vehicle/Field bucket recognises only $10,815.93. The remaining $6,110 sits in blank-bucket rows.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A116:G116"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A114:G114"/>
+    <mergeCell ref="A112:G112"/>
+    <mergeCell ref="A113:G113"/>
+    <mergeCell ref="A115:G115"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add gaps, data-quality defects and audit limitations tab
Second scrutiny pass. Records six gaps in the data (September 2025 and
January 2026 are near-empty months; the three Home Depot ledgers are
absent while $52,794.82 of Home Depot spend sits inside the two
trackers), six data-quality defects, six tests that came back clean, and
an explicit statement of what this audit cannot establish.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X9qK8zkdfoo6K5q1ScTX2U
</commit_message>
<xml_diff>
--- a/audit/Fuel_Auto_Fraud_Audit.xlsx
+++ b/audit/Fuel_Auto_Fraud_Audit.xlsx
@@ -8,25 +8,26 @@
   </bookViews>
   <sheets>
     <sheet name="13. Overhead Flagged + PAID" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="11. Fuel &amp; Auto vs Report" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="12. Flagged + PAID Status" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="1. Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="2. Flagged Transactions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="3. Full Fuel &amp; Auto Ledger" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="4. Vehicle Attribution" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="5. Job Attribution" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="6. Reconciliation" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="7. Auto Expenses Only" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="8. Auto by Company" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="9. Cap One Overhead F&amp;A" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="10. AmEx Overhead F&amp;A" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="14. Gaps &amp; Limitations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="11. Fuel &amp; Auto vs Report" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="12. Flagged + PAID Status" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="1. Summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2. Flagged Transactions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="3. Full Fuel &amp; Auto Ledger" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="4. Vehicle Attribution" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="5. Job Attribution" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="6. Reconciliation" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="7. Auto Expenses Only" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="8. Auto by Company" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="9. Cap One Overhead F&amp;A" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="10. AmEx Overhead F&amp;A" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'13. Overhead Flagged + PAID'!$A$43:$O$205</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'12. Flagged + PAID Status'!$A$26:$O$200</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'2. Flagged Transactions'!$A$1:$N$175</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'3. Full Fuel &amp; Auto Ledger'!$A$1:$N$241</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'7. Auto Expenses Only'!$A$19:$J$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'12. Flagged + PAID Status'!$A$26:$O$200</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'2. Flagged Transactions'!$A$1:$N$175</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'3. Full Fuel &amp; Auto Ledger'!$A$1:$N$241</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'7. Auto Expenses Only'!$A$19:$J$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -34,12 +35,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="$#,##0.00;($#,##0.00);-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="DD-MMM-YY"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -200,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -299,6 +299,18 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -11577,6 +11589,378 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>QUESTION 4 — RECONCILING THE $5,882 / $230 "FUEL &amp; AUTO" LINE</t>
+        </is>
+      </c>
+      <c r="B1" s="37" t="n"/>
+      <c r="C1" s="37" t="n"/>
+      <c r="D1" s="37" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Part A tests the reported tile against the trackers as they are categorised. Part B rebuilds the category from the transactions.</t>
+        </is>
+      </c>
+      <c r="B2" s="37" t="n"/>
+      <c r="C2" s="37" t="n"/>
+      <c r="D2" s="37" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="37" t="n"/>
+      <c r="B3" s="37" t="n"/>
+      <c r="C3" s="37" t="n"/>
+      <c r="D3" s="37" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>PART A — DOES THE REPORTED TILE TIE TO THE TRACKERS?</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>AmEx $</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Capital One $</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="40" t="inlineStr">
+        <is>
+          <t>Reported "Fuel &amp; Auto" tile</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>The figure on the category summary you sent</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="n">
+        <v>5882</v>
+      </c>
+      <c r="D6" s="41" t="n">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="37" t="inlineStr">
+        <is>
+          <t>Tracker Vehicle/Field bucket — Real Estate entity</t>
+        </is>
+      </c>
+      <c r="B7" s="37" t="inlineStr">
+        <is>
+          <t>Closest single slice in either workbook</t>
+        </is>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>6148.72</v>
+      </c>
+      <c r="D7" s="39" t="n">
+        <v>127.98</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="47" t="inlineStr">
+        <is>
+          <t>VARIANCE — tile vs closest slice</t>
+        </is>
+      </c>
+      <c r="B8" s="47" t="inlineStr">
+        <is>
+          <t>Not explained by any row or combination of rows</t>
+        </is>
+      </c>
+      <c r="C8" s="48" t="n">
+        <v>266.72</v>
+      </c>
+      <c r="D8" s="48" t="n">
+        <v>-102.02</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>Tracker Vehicle/Field bucket — all entities</t>
+        </is>
+      </c>
+      <c r="B9" s="37" t="inlineStr">
+        <is>
+          <t>Adds Matrix Group One, Peninsula Plumbing, Owner's Pay</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>10815.93</v>
+      </c>
+      <c r="D9" s="39" t="n">
+        <v>1990.03</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="37" t="n"/>
+      <c r="B10" s="37" t="n"/>
+      <c r="C10" s="37" t="n"/>
+      <c r="D10" s="37" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>PART B — REBUILDING FUEL &amp; AUTO FROM THE TRANSACTIONS</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Where it lives in the workbooks</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>AmEx $</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Capital One $</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>Correctly bucketed to Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>Overhead tabs, Bucket = Vehicle/Field</t>
+        </is>
+      </c>
+      <c r="C13" s="39" t="n">
+        <v>10078.55</v>
+      </c>
+      <c r="D13" s="39" t="n">
+        <v>1990.03</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="47" t="inlineStr">
+        <is>
+          <t>Uncategorised — Bucket left blank</t>
+        </is>
+      </c>
+      <c r="B14" s="47" t="inlineStr">
+        <is>
+          <t>Overhead tabs, no bucket assigned</t>
+        </is>
+      </c>
+      <c r="C14" s="48" t="n">
+        <v>6382.51</v>
+      </c>
+      <c r="D14" s="48" t="n">
+        <v>5495.26</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>Mis-bucketed to Travel / Meals</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t>Mexico fuel stops, 7-Eleven</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="n">
+        <v>464.81</v>
+      </c>
+      <c r="D15" s="41" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="40" t="inlineStr">
+        <is>
+          <t>Job-costed on the Property Expenses tabs</t>
+        </is>
+      </c>
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t>Never enters the overhead category rollup</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="n">
+        <v>2196.3</v>
+      </c>
+      <c r="D16" s="41" t="n">
+        <v>3518.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="61" t="inlineStr">
+        <is>
+          <t>TRUE FUEL &amp; AUTO EXPOSURE</t>
+        </is>
+      </c>
+      <c r="B17" s="61" t="inlineStr">
+        <is>
+          <t>De-duplicated; stale tabs excluded</t>
+        </is>
+      </c>
+      <c r="C17" s="62" t="n">
+        <v>19122.17</v>
+      </c>
+      <c r="D17" s="62" t="n">
+        <v>11003.79</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Understatement vs the reported tile</t>
+        </is>
+      </c>
+      <c r="B18" s="37" t="n"/>
+      <c r="C18" s="63" t="n">
+        <v>13240.17</v>
+      </c>
+      <c r="D18" s="63" t="n">
+        <v>10773.79</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Reported tile understates the category by a factor of</t>
+        </is>
+      </c>
+      <c r="B19" s="37" t="n"/>
+      <c r="C19" s="64" t="n">
+        <v>3.251</v>
+      </c>
+      <c r="D19" s="64" t="n">
+        <v>47.8426</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="37" t="n"/>
+      <c r="B20" s="37" t="n"/>
+      <c r="C20" s="37" t="n"/>
+      <c r="D20" s="37" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="59" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+      <c r="B21" s="37" t="n"/>
+      <c r="C21" s="37" t="n"/>
+      <c r="D21" s="37" t="n"/>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="60" t="inlineStr">
+        <is>
+          <t>•  The reported tile cannot be reproduced from either workbook. No row or combination of rows in the AmEx tracker sums to $5,882, and none in the Capital One tracker sums to $230. The closest categorised figures are $6,148.72 and $127.98 — a $266.72 shortfall on AmEx and a $102.02 overstatement on Capital One.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1">
+      <c r="A23" s="60" t="inlineStr">
+        <is>
+          <t>•  The tile also carries Home Depot 1511, 5253 and 8087 columns. Neither workbook supplied contains those card ledgers, so any Home Depot fuel or auto spend sits outside this audit entirely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="60" t="inlineStr">
+        <is>
+          <t>•  The single largest driver of the gap is uncategorised fuel: 90 AmEx charges and 27 Capital One charges carry a blank Bucket, so they never reach the Fuel &amp; Auto line even though they are plainly fuel, tolls or car washes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="60" t="inlineStr">
+        <is>
+          <t>•  Part B is measured on this audit's definition of fuel &amp; auto (fuel, tolls, fines, parking, car wash, DMV, towing, tyres/parts, vehicle upfit, car rental, transit). Part A uses the trackers' own Vehicle/Field bucket, which also contains items this audit classes elsewhere — the two are deliberately different measures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="60" t="inlineStr">
+        <is>
+          <t>•  Two stale tabs were excluded to avoid double counting: AmEx 'Overhead Expenses' (414 of its 421 rows repeat 'Copy of Overhead Expenses') and 'Copy of Capital One Business Pr' (a subset of 'Capital One Business Property E').</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="60" t="inlineStr">
+        <is>
+          <t>•  Bottom line: the tile shows $6,112 of combined Fuel &amp; Auto. Audited exposure across both cards is $30,125.96.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A24:D24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -15924,7 +16308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17202,7 +17586,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18664,7 +19048,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21676,6 +22060,718 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="75" t="inlineStr">
+        <is>
+          <t>GAPS, DATA QUALITY ISSUES, AND THE LIMITS OF THIS AUDIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Everything found on a second scrutiny pass, including the things this audit cannot tell you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>A. GAPS IN THE DATA — things that should be there and are not</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Exposure</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="86" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="B6" s="86" t="inlineStr">
+        <is>
+          <t>September 2025 has ZERO fuel &amp; auto charges on either card</t>
+        </is>
+      </c>
+      <c r="C6" s="86" t="inlineStr">
+        <is>
+          <t>August has 12 charges and October has 9. A whole month is blank. Either the cards genuinely went unused for 30 days, or a month of entries was never keyed in.</t>
+        </is>
+      </c>
+      <c r="D6" s="86" t="inlineStr">
+        <is>
+          <t>Unknown — a typical month runs $500-$2,500</t>
+        </is>
+      </c>
+      <c r="E6" s="86" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="86" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="B7" s="86" t="inlineStr">
+        <is>
+          <t>January 2026 has one charge, $135.00</t>
+        </is>
+      </c>
+      <c r="C7" s="86" t="inlineStr">
+        <is>
+          <t>December ran 15 charges, February ran 34. One entry for the whole of January is not credible.</t>
+        </is>
+      </c>
+      <c r="D7" s="86" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E7" s="86" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="86" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="B8" s="86" t="inlineStr">
+        <is>
+          <t>Home Depot cards are not in this audit at all</t>
+        </is>
+      </c>
+      <c r="C8" s="86" t="inlineStr">
+        <is>
+          <t>The report shows $21,472 unpaid across HD 1511 / 5253 / 8087. Neither workbook contains those ledgers.</t>
+        </is>
+      </c>
+      <c r="D8" s="86" t="inlineStr">
+        <is>
+          <t>$21,472 unreviewed</t>
+        </is>
+      </c>
+      <c r="E8" s="86" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="86" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="B9" s="86" t="inlineStr">
+        <is>
+          <t>Home Depot charges also appear INSIDE the two trackers</t>
+        </is>
+      </c>
+      <c r="C9" s="86" t="inlineStr">
+        <is>
+          <t>$52,794.82 of Home Depot spend is recorded in the AmEx and Capital One trackers. If the same purchases are also on the Home Depot card ledgers, the consolidated report double-counts them.</t>
+        </is>
+      </c>
+      <c r="D9" s="86" t="inlineStr">
+        <is>
+          <t>$52,794.82 at risk of double count</t>
+        </is>
+      </c>
+      <c r="E9" s="86" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="87" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="B10" s="87" t="inlineStr">
+        <is>
+          <t>No receipts, so no gallons</t>
+        </is>
+      </c>
+      <c r="C10" s="87" t="inlineStr">
+        <is>
+          <t>Every over-capacity finding is inferred from price, not proven from volume. A receipt showing gallons is what converts a flag into a fact.</t>
+        </is>
+      </c>
+      <c r="D10" s="87" t="inlineStr">
+        <is>
+          <t>Affects F2 ($318) and F3 ($1,138)</t>
+        </is>
+      </c>
+      <c r="E10" s="87" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="87" t="inlineStr">
+        <is>
+          <t>G6</t>
+        </is>
+      </c>
+      <c r="B11" s="87" t="inlineStr">
+        <is>
+          <t>No odometer or mileage log</t>
+        </is>
+      </c>
+      <c r="C11" s="87" t="inlineStr">
+        <is>
+          <t>Without miles driven there is no way to test whether fuel consumed is proportionate to work done.</t>
+        </is>
+      </c>
+      <c r="D11" s="87" t="inlineStr">
+        <is>
+          <t>Affects the whole audit</t>
+        </is>
+      </c>
+      <c r="E11" s="87" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>B. DATA QUALITY DEFECTS FOUND</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Defect</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="87" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B15" s="87" t="inlineStr">
+        <is>
+          <t>Four broken dates</t>
+        </is>
+      </c>
+      <c r="C15" s="87" t="inlineStr">
+        <is>
+          <t>"11/13/0105" (Starbucks, appears twice), "03//07/2026" (Amazon $1,203.11), and a cell holding two dates at once: "02/06/2026 02/07/2026" (Next Insurance $409.50)</t>
+        </is>
+      </c>
+      <c r="D15" s="87" t="inlineStr">
+        <is>
+          <t>$1,620.59</t>
+        </is>
+      </c>
+      <c r="E15" s="87" t="inlineStr">
+        <is>
+          <t>Fix the four cells</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="A16" s="87" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B16" s="87" t="inlineStr">
+        <is>
+          <t>Fuel &amp; auto on the AmEx tracker attributed to non-AmEx accounts</t>
+        </is>
+      </c>
+      <c r="C16" s="87" t="inlineStr">
+        <is>
+          <t>Rows on the AmEx tracker list the payer as Relay 5776, BOA 8217, Daliaz or Prescott Relay. Either the AmEx tracker is holding other cards' charges, or the payer field is wrong.</t>
+        </is>
+      </c>
+      <c r="D16" s="87" t="inlineStr">
+        <is>
+          <t>$881.87</t>
+        </is>
+      </c>
+      <c r="E16" s="87" t="inlineStr">
+        <is>
+          <t>Confirm which card actually paid</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
+      <c r="A17" s="87" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B17" s="87" t="inlineStr">
+        <is>
+          <t>31 rows marked "CANCELLED" but still carrying a charge</t>
+        </is>
+      </c>
+      <c r="C17" s="87" t="inlineStr">
+        <is>
+          <t>Recurring column says CANCELLED yet the amount stands. None are fuel or auto, but it is the same control weakness.</t>
+        </is>
+      </c>
+      <c r="D17" s="87" t="inlineStr">
+        <is>
+          <t>$3,274.56</t>
+        </is>
+      </c>
+      <c r="E17" s="87" t="inlineStr">
+        <is>
+          <t>Confirm the cancellations took effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="87" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B18" s="87" t="inlineStr">
+        <is>
+          <t>Two more near-duplicates my F1 test missed</t>
+        </is>
+      </c>
+      <c r="C18" s="87" t="inlineStr">
+        <is>
+          <t>Same amount on consecutive days with different vendor spellings: $100.00 A&amp;A Gas on 29-Jun and 30-Jun; $38.00 Parking Citation on 14-Oct and 15-Oct. F1 only matches same-day.</t>
+        </is>
+      </c>
+      <c r="D18" s="87" t="inlineStr">
+        <is>
+          <t>$138.00</t>
+        </is>
+      </c>
+      <c r="E18" s="87" t="inlineStr">
+        <is>
+          <t>Check against the statements</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="52" customHeight="1">
+      <c r="A19" s="87" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B19" s="87" t="inlineStr">
+        <is>
+          <t>118 refunds and credits across the workbooks</t>
+        </is>
+      </c>
+      <c r="C19" s="87" t="inlineStr">
+        <is>
+          <t>Totalling -$32,755.78, including a $4,278.28 Apple Store credit and a $2,816.00 insurance credit. Only one is in fuel &amp; auto (-$2.05 Clipper). Large credits should be matched to the original charges.</t>
+        </is>
+      </c>
+      <c r="D19" s="87" t="inlineStr">
+        <is>
+          <t>-$32,755.78</t>
+        </is>
+      </c>
+      <c r="E19" s="87" t="inlineStr">
+        <is>
+          <t>Verify each credit ties to a charge</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="52" customHeight="1">
+      <c r="A20" s="87" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B20" s="87" t="inlineStr">
+        <is>
+          <t>Capital One overhead is spread across four overlapping tabs</t>
+        </is>
+      </c>
+      <c r="C20" s="87" t="inlineStr">
+        <is>
+          <t>Personal Overhead, Business - Overhead, Overhead Expenses and PPS Expenses all hold February 2026 data with no key linking them. This is the structural cause of the duplicate postings.</t>
+        </is>
+      </c>
+      <c r="D20" s="87" t="inlineStr">
+        <is>
+          <t>Caused $2,296.16 of duplicates</t>
+        </is>
+      </c>
+      <c r="E20" s="87" t="inlineStr">
+        <is>
+          <t>Consolidate to one tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>C. THINGS I CHECKED THAT CAME BACK CLEAN</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="88" t="inlineStr">
+        <is>
+          <t>Fuel vendors with a missing amount</t>
+        </is>
+      </c>
+      <c r="B24" s="88" t="inlineStr">
+        <is>
+          <t>None. No fuel charge is invisible to the totals for want of a figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="88" t="inlineStr">
+        <is>
+          <t>Fuel hiding in tabs outside the audit scope</t>
+        </is>
+      </c>
+      <c r="B25" s="88" t="inlineStr">
+        <is>
+          <t>$2,705.33 found, and all of it is on the two stale duplicate tabs already excluded. Nothing was missed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="88" t="inlineStr">
+        <is>
+          <t>Overhead charges that actually name a property</t>
+        </is>
+      </c>
+      <c r="B26" s="88" t="inlineStr">
+        <is>
+          <t>None. The overhead / property split is applied consistently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="88" t="inlineStr">
+        <is>
+          <t>Property-tab fuel with the job left blank</t>
+        </is>
+      </c>
+      <c r="B27" s="88" t="inlineStr">
+        <is>
+          <t>None. Job-costed fuel is properly tagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="88" t="inlineStr">
+        <is>
+          <t>Weekend fuel concentration</t>
+        </is>
+      </c>
+      <c r="B28" s="88" t="inlineStr">
+        <is>
+          <t>22% of fuel spend falls on a weekend, spread evenly across Saturday and Sunday. That is normal for a field business and is NOT a finding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="88" t="inlineStr">
+        <is>
+          <t>Cancelled subscriptions among fuel/auto vendors</t>
+        </is>
+      </c>
+      <c r="B29" s="88" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>D. WHAT THIS AUDIT CANNOT TELL YOU — read before acting on any finding</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+    </row>
+    <row r="32" ht="44" customHeight="1">
+      <c r="A32" s="60" t="inlineStr">
+        <is>
+          <t>•  A flag is not proof. It means the charge does not look like ordinary fleet use and needs a receipt, a fuel log or an explanation. Most will clear. F1 duplicates are the exception — a duplicate is a fact, not an inference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="44" customHeight="1">
+      <c r="A33" s="60" t="inlineStr">
+        <is>
+          <t>•  The $140 tank-capacity threshold is my estimate, built from a 24-gallon ProMaster at roughly $4.50-$5.00 a gallon. If the fleet includes a larger tank, or if someone legitimately fills two vehicles on one card, some F2 findings will clear. Receipts settle it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1">
+      <c r="A34" s="60" t="inlineStr">
+        <is>
+          <t>•  I never saw a card statement. Everything here is measured against the trackers, so if a charge was never entered into a tracker, this audit cannot see it. The September 2025 gap is exactly that risk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="44" customHeight="1">
+      <c r="A35" s="60" t="inlineStr">
+        <is>
+          <t>•  I do not know who drives which vehicle. Driver names come from what someone typed into a description field, and only 8 charges name anyone at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="44" customHeight="1">
+      <c r="A36" s="60" t="inlineStr">
+        <is>
+          <t>•  The PAID flags are as at the file I was given (data through 29-Jul-2026). Your accounting report ran 01-Aug-2026 and disagrees. Anything sliced by PAID status inherits that uncertainty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="44" customHeight="1">
+      <c r="A37" s="60" t="inlineStr">
+        <is>
+          <t>•  Fuel prices moved over the period. A $95 fill in August 2025 and a $95 fill in July 2026 are not the same number of gallons, and I have not price-adjusted anything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="44" customHeight="1">
+      <c r="A38" s="60" t="inlineStr">
+        <is>
+          <t>•  I classified charges by vendor name and description text. A miscoded or blank description can put a charge in the wrong category — which is itself finding F8, so the classification and the defect are entangled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>E. WHAT I WOULD ASK FOR NEXT, IN ORDER</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="5" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Why it matters most</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="46" customHeight="1">
+      <c r="A42" s="89" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B42" s="89" t="inlineStr">
+        <is>
+          <t>The three Home Depot card ledgers</t>
+        </is>
+      </c>
+      <c r="C42" s="89" t="inlineStr">
+        <is>
+          <t>$21,472 of unpaid balance is completely unreviewed, and $52,794.82 of Home Depot spend already sits in the two trackers — the overlap has to be resolved before any consolidated number is trustworthy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="46" customHeight="1">
+      <c r="A43" s="89" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B43" s="89" t="inlineStr">
+        <is>
+          <t>September 2025 and January 2026 card statements</t>
+        </is>
+      </c>
+      <c r="C43" s="89" t="inlineStr">
+        <is>
+          <t>Two near-empty months. If charges exist that were never entered, every total in this audit is understated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="46" customHeight="1">
+      <c r="A44" s="89" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B44" s="89" t="inlineStr">
+        <is>
+          <t>Merchant receipts for the 13 flagged fills</t>
+        </is>
+      </c>
+      <c r="C44" s="89" t="inlineStr">
+        <is>
+          <t>The 2 over-capacity and 11 round-dollar charges in Overhead. Receipts show gallons, which is the only thing that turns these from suspicion into fact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="46" customHeight="1">
+      <c r="A45" s="89" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B45" s="89" t="inlineStr">
+        <is>
+          <t>The FasTrak transponder statement</t>
+        </is>
+      </c>
+      <c r="C45" s="89" t="inlineStr">
+        <is>
+          <t>One document explains $4,397.95 of tolls and fines, and it lists the plate and crossing time for every charge — which also answers "which vehicle" for that whole block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="46" customHeight="1">
+      <c r="A46" s="89" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B46" s="89" t="inlineStr">
+        <is>
+          <t>The transaction-level export behind the 01-Aug accounting report</t>
+        </is>
+      </c>
+      <c r="C46" s="89" t="inlineStr">
+        <is>
+          <t>The only way to reconcile the $5,882 / $230 and find the $2,646 difference.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A36:E36"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -24748,7 +25844,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -34395,7 +35491,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -35141,7 +36237,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -43446,7 +44542,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -54611,7 +55707,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -55222,7 +56318,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -58596,376 +59692,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="36" t="inlineStr">
-        <is>
-          <t>QUESTION 4 — RECONCILING THE $5,882 / $230 "FUEL &amp; AUTO" LINE</t>
-        </is>
-      </c>
-      <c r="B1" s="37" t="n"/>
-      <c r="C1" s="37" t="n"/>
-      <c r="D1" s="37" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Part A tests the reported tile against the trackers as they are categorised. Part B rebuilds the category from the transactions.</t>
-        </is>
-      </c>
-      <c r="B2" s="37" t="n"/>
-      <c r="C2" s="37" t="n"/>
-      <c r="D2" s="37" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="37" t="n"/>
-      <c r="B3" s="37" t="n"/>
-      <c r="C3" s="37" t="n"/>
-      <c r="D3" s="37" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>PART A — DOES THE REPORTED TILE TIE TO THE TRACKERS?</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Measure</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Definition</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>AmEx $</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Capital One $</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="40" t="inlineStr">
-        <is>
-          <t>Reported "Fuel &amp; Auto" tile</t>
-        </is>
-      </c>
-      <c r="B6" s="40" t="inlineStr">
-        <is>
-          <t>The figure on the category summary you sent</t>
-        </is>
-      </c>
-      <c r="C6" s="41" t="n">
-        <v>5882</v>
-      </c>
-      <c r="D6" s="41" t="n">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="37" t="inlineStr">
-        <is>
-          <t>Tracker Vehicle/Field bucket — Real Estate entity</t>
-        </is>
-      </c>
-      <c r="B7" s="37" t="inlineStr">
-        <is>
-          <t>Closest single slice in either workbook</t>
-        </is>
-      </c>
-      <c r="C7" s="39" t="n">
-        <v>6148.72</v>
-      </c>
-      <c r="D7" s="39" t="n">
-        <v>127.98</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="47" t="inlineStr">
-        <is>
-          <t>VARIANCE — tile vs closest slice</t>
-        </is>
-      </c>
-      <c r="B8" s="47" t="inlineStr">
-        <is>
-          <t>Not explained by any row or combination of rows</t>
-        </is>
-      </c>
-      <c r="C8" s="48" t="n">
-        <v>266.72</v>
-      </c>
-      <c r="D8" s="48" t="n">
-        <v>-102.02</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="37" t="inlineStr">
-        <is>
-          <t>Tracker Vehicle/Field bucket — all entities</t>
-        </is>
-      </c>
-      <c r="B9" s="37" t="inlineStr">
-        <is>
-          <t>Adds Matrix Group One, Peninsula Plumbing, Owner's Pay</t>
-        </is>
-      </c>
-      <c r="C9" s="39" t="n">
-        <v>10815.93</v>
-      </c>
-      <c r="D9" s="39" t="n">
-        <v>1990.03</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="37" t="n"/>
-      <c r="B10" s="37" t="n"/>
-      <c r="C10" s="37" t="n"/>
-      <c r="D10" s="37" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>PART B — REBUILDING FUEL &amp; AUTO FROM THE TRANSACTIONS</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Where it lives in the workbooks</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>AmEx $</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Capital One $</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="37" t="inlineStr">
-        <is>
-          <t>Correctly bucketed to Vehicle/Field</t>
-        </is>
-      </c>
-      <c r="B13" s="37" t="inlineStr">
-        <is>
-          <t>Overhead tabs, Bucket = Vehicle/Field</t>
-        </is>
-      </c>
-      <c r="C13" s="39" t="n">
-        <v>10078.55</v>
-      </c>
-      <c r="D13" s="39" t="n">
-        <v>1990.03</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="47" t="inlineStr">
-        <is>
-          <t>Uncategorised — Bucket left blank</t>
-        </is>
-      </c>
-      <c r="B14" s="47" t="inlineStr">
-        <is>
-          <t>Overhead tabs, no bucket assigned</t>
-        </is>
-      </c>
-      <c r="C14" s="48" t="n">
-        <v>6382.51</v>
-      </c>
-      <c r="D14" s="48" t="n">
-        <v>5495.26</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="40" t="inlineStr">
-        <is>
-          <t>Mis-bucketed to Travel / Meals</t>
-        </is>
-      </c>
-      <c r="B15" s="40" t="inlineStr">
-        <is>
-          <t>Mexico fuel stops, 7-Eleven</t>
-        </is>
-      </c>
-      <c r="C15" s="41" t="n">
-        <v>464.81</v>
-      </c>
-      <c r="D15" s="41" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="40" t="inlineStr">
-        <is>
-          <t>Job-costed on the Property Expenses tabs</t>
-        </is>
-      </c>
-      <c r="B16" s="40" t="inlineStr">
-        <is>
-          <t>Never enters the overhead category rollup</t>
-        </is>
-      </c>
-      <c r="C16" s="41" t="n">
-        <v>2196.3</v>
-      </c>
-      <c r="D16" s="41" t="n">
-        <v>3518.5</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="61" t="inlineStr">
-        <is>
-          <t>TRUE FUEL &amp; AUTO EXPOSURE</t>
-        </is>
-      </c>
-      <c r="B17" s="61" t="inlineStr">
-        <is>
-          <t>De-duplicated; stale tabs excluded</t>
-        </is>
-      </c>
-      <c r="C17" s="62" t="n">
-        <v>19122.17</v>
-      </c>
-      <c r="D17" s="62" t="n">
-        <v>11003.79</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>Understatement vs the reported tile</t>
-        </is>
-      </c>
-      <c r="B18" s="37" t="n"/>
-      <c r="C18" s="63" t="n">
-        <v>13240.17</v>
-      </c>
-      <c r="D18" s="63" t="n">
-        <v>10773.79</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>Reported tile understates the category by a factor of</t>
-        </is>
-      </c>
-      <c r="B19" s="37" t="n"/>
-      <c r="C19" s="64" t="n">
-        <v>3.251</v>
-      </c>
-      <c r="D19" s="64" t="n">
-        <v>47.8426</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="37" t="n"/>
-      <c r="B20" s="37" t="n"/>
-      <c r="C20" s="37" t="n"/>
-      <c r="D20" s="37" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="59" t="inlineStr">
-        <is>
-          <t>NOTES</t>
-        </is>
-      </c>
-      <c r="B21" s="37" t="n"/>
-      <c r="C21" s="37" t="n"/>
-      <c r="D21" s="37" t="n"/>
-    </row>
-    <row r="22" ht="42" customHeight="1">
-      <c r="A22" s="60" t="inlineStr">
-        <is>
-          <t>•  The reported tile cannot be reproduced from either workbook. No row or combination of rows in the AmEx tracker sums to $5,882, and none in the Capital One tracker sums to $230. The closest categorised figures are $6,148.72 and $127.98 — a $266.72 shortfall on AmEx and a $102.02 overstatement on Capital One.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="60" t="inlineStr">
-        <is>
-          <t>•  The tile also carries Home Depot 1511, 5253 and 8087 columns. Neither workbook supplied contains those card ledgers, so any Home Depot fuel or auto spend sits outside this audit entirely.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="42" customHeight="1">
-      <c r="A24" s="60" t="inlineStr">
-        <is>
-          <t>•  The single largest driver of the gap is uncategorised fuel: 90 AmEx charges and 27 Capital One charges carry a blank Bucket, so they never reach the Fuel &amp; Auto line even though they are plainly fuel, tolls or car washes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="42" customHeight="1">
-      <c r="A25" s="60" t="inlineStr">
-        <is>
-          <t>•  Part B is measured on this audit's definition of fuel &amp; auto (fuel, tolls, fines, parking, car wash, DMV, towing, tyres/parts, vehicle upfit, car rental, transit). Part A uses the trackers' own Vehicle/Field bucket, which also contains items this audit classes elsewhere — the two are deliberately different measures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="42" customHeight="1">
-      <c r="A26" s="60" t="inlineStr">
-        <is>
-          <t>•  Two stale tabs were excluded to avoid double counting: AmEx 'Overhead Expenses' (414 of its 421 rows repeat 'Copy of Overhead Expenses') and 'Copy of Capital One Business Pr' (a subset of 'Capital One Business Property E').</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="42" customHeight="1">
-      <c r="A27" s="60" t="inlineStr">
-        <is>
-          <t>•  Bottom line: the tile shows $6,112 of combined Fuel &amp; Auto. Audited exposure across both cards is $30,125.96.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A24:D24"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>